<commit_message>
Add domain suggestions for all 126 individual sites and 26 bundle hubs
Unique brand token per site following fleet naming conventions; all
suggested domains returned NXDOMAIN on DNS check. doorfix-locksmiths.co.uk
(already owned) is assigned to Bundle 01.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018qYwdxW5238hQ6ii9dUE6c
</commit_message>
<xml_diff>
--- a/data/locksmith-fleet/coverage-plan-final.xlsx
+++ b/data/locksmith-fleet/coverage-plan-final.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master Plan'!$A$1:$L$408</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master Plan'!$A$1:$M$408</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -72,7 +72,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -85,6 +85,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -450,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L408"/>
+  <dimension ref="A1:M408"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -465,6 +466,7 @@
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="9" customWidth="1" min="11" max="11"/>
     <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="42" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -528,6 +530,11 @@
           <t>Competing Live Subdomain</t>
         </is>
       </c>
+      <c r="M1" s="8" t="inlineStr">
+        <is>
+          <t>Suggested Domain</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -802,6 +809,11 @@
           <t>loughborough.surelok-locksmiths.co.uk</t>
         </is>
       </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>boltrouteloughboroughlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1120,6 +1132,11 @@
           <t>hemelhempstead.surelok-locksmiths.co.uk</t>
         </is>
       </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>keycorehemelhempsteadlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1262,6 +1279,11 @@
           <t>peterborough.shieldx-locksmiths.co.uk</t>
         </is>
       </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>boltwavepeterboroughlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1314,6 +1336,11 @@
       <c r="L18" s="4" t="inlineStr">
         <is>
           <t>stalbans.toplock-locksmiths.co.uk</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>keyqueststalbanslocksmiths.co.uk</t>
         </is>
       </c>
     </row>
@@ -1634,6 +1661,11 @@
           <t>gateshead.suresec-locksmiths.co.uk</t>
         </is>
       </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>latchmaxgatesheadlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1776,6 +1808,11 @@
           <t>sunderland.boltlok-locksmiths.co.uk</t>
         </is>
       </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>keypointsunderlandlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1962,6 +1999,11 @@
           <t>chester.shield-locksmiths.co.uk</t>
         </is>
       </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>keygridchesterlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2368,6 +2410,11 @@
           <t>rochdale.toplock-locksmiths.co.uk</t>
         </is>
       </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>lockcrewrochdalelocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -2422,6 +2469,11 @@
           <t>runcorn.shield-locksmiths.co.uk</t>
         </is>
       </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>boltsmartruncornlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -2476,6 +2528,11 @@
           <t>wallasey.boltpro-locksmiths.co.uk</t>
         </is>
       </c>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>lockjetwallaseylocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -2528,6 +2585,11 @@
       <c r="L44" s="4" t="inlineStr">
         <is>
           <t>warrington.boltman-locksmiths.co.uk</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>boltpeakwarringtonlocksmiths.co.uk</t>
         </is>
       </c>
     </row>
@@ -2760,6 +2822,11 @@
           <t>aylesbury.boltman-locksmiths.co.uk</t>
         </is>
       </c>
+      <c r="M49" s="2" t="inlineStr">
+        <is>
+          <t>bolthavenaylesburylocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3034,6 +3101,11 @@
           <t>farnborough.shieldx-locksmiths.co.uk</t>
         </is>
       </c>
+      <c r="M55" s="2" t="inlineStr">
+        <is>
+          <t>latchsmartfarnboroughlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3176,6 +3248,11 @@
           <t>hastings.shieldx-locksmiths.co.uk</t>
         </is>
       </c>
+      <c r="M58" s="2" t="inlineStr">
+        <is>
+          <t>boltgridhastingslocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -3406,6 +3483,11 @@
           <t>oxford.boltfix-locksmiths.co.uk</t>
         </is>
       </c>
+      <c r="M63" s="2" t="inlineStr">
+        <is>
+          <t>latchpeakoxfordlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -3504,6 +3586,11 @@
           <t>slough.boltpro-locksmiths.co.uk</t>
         </is>
       </c>
+      <c r="M65" s="2" t="inlineStr">
+        <is>
+          <t>lockpointsloughlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -3646,6 +3733,11 @@
           <t>woking.trulock-locksmiths.co.uk</t>
         </is>
       </c>
+      <c r="M68" s="2" t="inlineStr">
+        <is>
+          <t>latchpulsewokinglocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
@@ -3700,6 +3792,11 @@
           <t>worthing.trulock-locksmiths.co.uk</t>
         </is>
       </c>
+      <c r="M69" s="2" t="inlineStr">
+        <is>
+          <t>keycrewworthinglocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
@@ -3752,6 +3849,11 @@
       <c r="L70" s="4" t="inlineStr">
         <is>
           <t>bournemouth.shield-locksmiths.co.uk</t>
+        </is>
+      </c>
+      <c r="M70" s="2" t="inlineStr">
+        <is>
+          <t>lockwavebournemouthlocksmiths.co.uk</t>
         </is>
       </c>
     </row>
@@ -3896,6 +3998,11 @@
           <t>cheltenham.steelok-locksmiths.co.uk</t>
         </is>
       </c>
+      <c r="M73" s="2" t="inlineStr">
+        <is>
+          <t>lockmaxcheltenhamlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -4214,6 +4321,11 @@
           <t>burtonupontrent.steelok-locksmiths.co.uk</t>
         </is>
       </c>
+      <c r="M80" s="2" t="inlineStr">
+        <is>
+          <t>lockpulseburtonontrentlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -4488,6 +4600,11 @@
           <t>stoke-on-trent.surelok-locksmiths.co.uk</t>
         </is>
       </c>
+      <c r="M86" s="2" t="inlineStr">
+        <is>
+          <t>latchstarstokeontrentlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
@@ -4540,6 +4657,11 @@
       <c r="L87" s="4" t="inlineStr">
         <is>
           <t>tamworth.suresec-locksmiths.co.uk</t>
+        </is>
+      </c>
+      <c r="M87" s="2" t="inlineStr">
+        <is>
+          <t>boltpulsetamworthlocksmiths.co.uk</t>
         </is>
       </c>
     </row>
@@ -4816,6 +4938,11 @@
           <t>doncaster.boltfix-locksmiths.co.uk</t>
         </is>
       </c>
+      <c r="M93" s="2" t="inlineStr">
+        <is>
+          <t>latchhavendoncasterlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
@@ -4868,6 +4995,11 @@
       <c r="L94" s="4" t="inlineStr">
         <is>
           <t>grimsby.boltlok-locksmiths.co.uk</t>
+        </is>
+      </c>
+      <c r="M94" s="2" t="inlineStr">
+        <is>
+          <t>keyjetgrimsbylocksmiths.co.uk</t>
         </is>
       </c>
     </row>
@@ -5180,6 +5312,11 @@
       </c>
       <c r="K101" s="2" t="inlineStr"/>
       <c r="L101" s="2" t="inlineStr"/>
+      <c r="M101" s="2" t="inlineStr">
+        <is>
+          <t>keypulsechesterfieldlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -5226,6 +5363,11 @@
       </c>
       <c r="K102" s="2" t="inlineStr"/>
       <c r="L102" s="2" t="inlineStr"/>
+      <c r="M102" s="2" t="inlineStr">
+        <is>
+          <t>lockstarderbylocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -5272,6 +5414,11 @@
       </c>
       <c r="K103" s="2" t="inlineStr"/>
       <c r="L103" s="2" t="inlineStr"/>
+      <c r="M103" s="2" t="inlineStr">
+        <is>
+          <t>keyzonenorthamptonlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -5318,6 +5465,11 @@
       </c>
       <c r="K104" s="2" t="inlineStr"/>
       <c r="L104" s="2" t="inlineStr"/>
+      <c r="M104" s="2" t="inlineStr">
+        <is>
+          <t>boltmaxbasildonlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -5364,6 +5516,11 @@
       </c>
       <c r="K105" s="2" t="inlineStr"/>
       <c r="L105" s="2" t="inlineStr"/>
+      <c r="M105" s="2" t="inlineStr">
+        <is>
+          <t>latchedgebedfordlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -5410,6 +5567,11 @@
       </c>
       <c r="K106" s="2" t="inlineStr"/>
       <c r="L106" s="2" t="inlineStr"/>
+      <c r="M106" s="2" t="inlineStr">
+        <is>
+          <t>boltspotbraintreelocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -5456,6 +5618,11 @@
       </c>
       <c r="K107" s="2" t="inlineStr"/>
       <c r="L107" s="2" t="inlineStr"/>
+      <c r="M107" s="2" t="inlineStr">
+        <is>
+          <t>keylinecambridgelocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -5502,6 +5669,11 @@
       </c>
       <c r="K108" s="2" t="inlineStr"/>
       <c r="L108" s="2" t="inlineStr"/>
+      <c r="M108" s="2" t="inlineStr">
+        <is>
+          <t>latchcrewchelmsfordlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -5548,6 +5720,11 @@
       </c>
       <c r="K109" s="2" t="inlineStr"/>
       <c r="L109" s="2" t="inlineStr"/>
+      <c r="M109" s="2" t="inlineStr">
+        <is>
+          <t>latchlinkcolchesterlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -5594,6 +5771,11 @@
       </c>
       <c r="K110" s="2" t="inlineStr"/>
       <c r="L110" s="2" t="inlineStr"/>
+      <c r="M110" s="2" t="inlineStr">
+        <is>
+          <t>lockgateharlowlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -5640,6 +5822,11 @@
       </c>
       <c r="K111" s="2" t="inlineStr"/>
       <c r="L111" s="2" t="inlineStr"/>
+      <c r="M111" s="2" t="inlineStr">
+        <is>
+          <t>locklineipswichlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -5686,6 +5873,11 @@
       </c>
       <c r="K112" s="2" t="inlineStr"/>
       <c r="L112" s="2" t="inlineStr"/>
+      <c r="M112" s="2" t="inlineStr">
+        <is>
+          <t>boltzonelutonlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -5732,6 +5924,11 @@
       </c>
       <c r="K113" s="2" t="inlineStr"/>
       <c r="L113" s="2" t="inlineStr"/>
+      <c r="M113" s="2" t="inlineStr">
+        <is>
+          <t>lockpeaksouthendlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -5778,6 +5975,11 @@
       </c>
       <c r="K114" s="2" t="inlineStr"/>
       <c r="L114" s="2" t="inlineStr"/>
+      <c r="M114" s="2" t="inlineStr">
+        <is>
+          <t>boltcorestevenagelocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -5824,6 +6026,11 @@
       </c>
       <c r="K115" s="2" t="inlineStr"/>
       <c r="L115" s="2" t="inlineStr"/>
+      <c r="M115" s="2" t="inlineStr">
+        <is>
+          <t>latchgatedarlingtonlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -5870,6 +6077,11 @@
       </c>
       <c r="K116" s="2" t="inlineStr"/>
       <c r="L116" s="2" t="inlineStr"/>
+      <c r="M116" s="2" t="inlineStr">
+        <is>
+          <t>lockhavenhartlepoollocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -5916,6 +6128,11 @@
       </c>
       <c r="K117" s="2" t="inlineStr"/>
       <c r="L117" s="2" t="inlineStr"/>
+      <c r="M117" s="2" t="inlineStr">
+        <is>
+          <t>boltlinemiddlesbroughlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -5962,6 +6179,11 @@
       </c>
       <c r="K118" s="2" t="inlineStr"/>
       <c r="L118" s="2" t="inlineStr"/>
+      <c r="M118" s="2" t="inlineStr">
+        <is>
+          <t>keystarnewcastlelocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -6008,6 +6230,11 @@
       </c>
       <c r="K119" s="2" t="inlineStr"/>
       <c r="L119" s="2" t="inlineStr"/>
+      <c r="M119" s="2" t="inlineStr">
+        <is>
+          <t>boltjetstocktonlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -6054,6 +6281,11 @@
       </c>
       <c r="K120" s="2" t="inlineStr"/>
       <c r="L120" s="2" t="inlineStr"/>
+      <c r="M120" s="2" t="inlineStr">
+        <is>
+          <t>latchwaveboltonlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -6100,6 +6332,11 @@
       </c>
       <c r="K121" s="2" t="inlineStr"/>
       <c r="L121" s="2" t="inlineStr"/>
+      <c r="M121" s="2" t="inlineStr">
+        <is>
+          <t>keysprintchorleylocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -6146,6 +6383,11 @@
       </c>
       <c r="K122" s="2" t="inlineStr"/>
       <c r="L122" s="2" t="inlineStr"/>
+      <c r="M122" s="2" t="inlineStr">
+        <is>
+          <t>boltcrewoldhamlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -6192,6 +6434,11 @@
       </c>
       <c r="K123" s="2" t="inlineStr"/>
       <c r="L123" s="2" t="inlineStr"/>
+      <c r="M123" s="2" t="inlineStr">
+        <is>
+          <t>lockcoreprestonlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -6238,6 +6485,11 @@
       </c>
       <c r="K124" s="2" t="inlineStr"/>
       <c r="L124" s="2" t="inlineStr"/>
+      <c r="M124" s="2" t="inlineStr">
+        <is>
+          <t>latchcraftsalfordlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -6284,6 +6536,11 @@
       </c>
       <c r="K125" s="2" t="inlineStr"/>
       <c r="L125" s="2" t="inlineStr"/>
+      <c r="M125" s="2" t="inlineStr">
+        <is>
+          <t>latchmatestockportlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -6330,6 +6587,11 @@
       </c>
       <c r="K126" s="2" t="inlineStr"/>
       <c r="L126" s="2" t="inlineStr"/>
+      <c r="M126" s="2" t="inlineStr">
+        <is>
+          <t>latchkingwiganlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -6376,6 +6638,11 @@
       </c>
       <c r="K127" s="2" t="inlineStr"/>
       <c r="L127" s="2" t="inlineStr"/>
+      <c r="M127" s="2" t="inlineStr">
+        <is>
+          <t>lockkingashfordlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -6422,6 +6689,11 @@
       </c>
       <c r="K128" s="2" t="inlineStr"/>
       <c r="L128" s="2" t="inlineStr"/>
+      <c r="M128" s="2" t="inlineStr">
+        <is>
+          <t>boltsparkcanterburylocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -6468,6 +6740,11 @@
       </c>
       <c r="K129" s="2" t="inlineStr"/>
       <c r="L129" s="2" t="inlineStr"/>
+      <c r="M129" s="2" t="inlineStr">
+        <is>
+          <t>lockmatecrawleylocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -6514,6 +6791,11 @@
       </c>
       <c r="K130" s="2" t="inlineStr"/>
       <c r="L130" s="2" t="inlineStr"/>
+      <c r="M130" s="2" t="inlineStr">
+        <is>
+          <t>boltsprintdoverlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -6560,6 +6842,11 @@
       </c>
       <c r="K131" s="2" t="inlineStr"/>
       <c r="L131" s="2" t="inlineStr"/>
+      <c r="M131" s="2" t="inlineStr">
+        <is>
+          <t>keyedgeeastbournelocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -6606,6 +6893,11 @@
       </c>
       <c r="K132" s="2" t="inlineStr"/>
       <c r="L132" s="2" t="inlineStr"/>
+      <c r="M132" s="2" t="inlineStr">
+        <is>
+          <t>latchspotfarehamlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -6652,6 +6944,11 @@
       </c>
       <c r="K133" s="2" t="inlineStr"/>
       <c r="L133" s="2" t="inlineStr"/>
+      <c r="M133" s="2" t="inlineStr">
+        <is>
+          <t>boltcraftgillinghamlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -6698,6 +6995,11 @@
       </c>
       <c r="K134" s="2" t="inlineStr"/>
       <c r="L134" s="2" t="inlineStr"/>
+      <c r="M134" s="2" t="inlineStr">
+        <is>
+          <t>locknestguildfordlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -6744,6 +7046,11 @@
       </c>
       <c r="K135" s="2" t="inlineStr"/>
       <c r="L135" s="2" t="inlineStr"/>
+      <c r="M135" s="2" t="inlineStr">
+        <is>
+          <t>keyspothorshamlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -6790,6 +7097,11 @@
       </c>
       <c r="K136" s="2" t="inlineStr"/>
       <c r="L136" s="2" t="inlineStr"/>
+      <c r="M136" s="2" t="inlineStr">
+        <is>
+          <t>lockcraftmaidstonelocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -6836,6 +7148,11 @@
       </c>
       <c r="K137" s="2" t="inlineStr"/>
       <c r="L137" s="2" t="inlineStr"/>
+      <c r="M137" s="2" t="inlineStr">
+        <is>
+          <t>keywavemiltonkeyneslocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -6882,6 +7199,11 @@
       </c>
       <c r="K138" s="2" t="inlineStr"/>
       <c r="L138" s="2" t="inlineStr"/>
+      <c r="M138" s="2" t="inlineStr">
+        <is>
+          <t>latchzonereadinglocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -6928,6 +7250,11 @@
       </c>
       <c r="K139" s="2" t="inlineStr"/>
       <c r="L139" s="2" t="inlineStr"/>
+      <c r="M139" s="2" t="inlineStr">
+        <is>
+          <t>lockspotwinchesterlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -6974,6 +7301,11 @@
       </c>
       <c r="K140" s="2" t="inlineStr"/>
       <c r="L140" s="2" t="inlineStr"/>
+      <c r="M140" s="2" t="inlineStr">
+        <is>
+          <t>latchsparkwokinghamlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -7020,6 +7352,11 @@
       </c>
       <c r="K141" s="2" t="inlineStr"/>
       <c r="L141" s="2" t="inlineStr"/>
+      <c r="M141" s="2" t="inlineStr">
+        <is>
+          <t>keygatebathlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -7066,6 +7403,11 @@
       </c>
       <c r="K142" s="2" t="inlineStr"/>
       <c r="L142" s="2" t="inlineStr"/>
+      <c r="M142" s="2" t="inlineStr">
+        <is>
+          <t>boltmategloucesterlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -7112,6 +7454,11 @@
       </c>
       <c r="K143" s="2" t="inlineStr"/>
       <c r="L143" s="2" t="inlineStr"/>
+      <c r="M143" s="2" t="inlineStr">
+        <is>
+          <t>locklinkpoolelocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -7158,6 +7505,11 @@
       </c>
       <c r="K144" s="2" t="inlineStr"/>
       <c r="L144" s="2" t="inlineStr"/>
+      <c r="M144" s="2" t="inlineStr">
+        <is>
+          <t>locksquadstroudlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -7204,6 +7556,11 @@
       </c>
       <c r="K145" s="2" t="inlineStr"/>
       <c r="L145" s="2" t="inlineStr"/>
+      <c r="M145" s="2" t="inlineStr">
+        <is>
+          <t>latchjetwestonsupermarelocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -7250,6 +7607,11 @@
       </c>
       <c r="K146" s="2" t="inlineStr"/>
       <c r="L146" s="2" t="inlineStr"/>
+      <c r="M146" s="2" t="inlineStr">
+        <is>
+          <t>latchroutedudleylocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -7296,6 +7658,11 @@
       </c>
       <c r="K147" s="2" t="inlineStr"/>
       <c r="L147" s="2" t="inlineStr"/>
+      <c r="M147" s="2" t="inlineStr">
+        <is>
+          <t>latchsprintlichfieldlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -7342,6 +7709,11 @@
       </c>
       <c r="K148" s="2" t="inlineStr"/>
       <c r="L148" s="2" t="inlineStr"/>
+      <c r="M148" s="2" t="inlineStr">
+        <is>
+          <t>latchnestnewcastleunderlymelocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -7388,6 +7760,11 @@
       </c>
       <c r="K149" s="2" t="inlineStr"/>
       <c r="L149" s="2" t="inlineStr"/>
+      <c r="M149" s="2" t="inlineStr">
+        <is>
+          <t>boltkingredditchlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -7434,6 +7811,11 @@
       </c>
       <c r="K150" s="2" t="inlineStr"/>
       <c r="L150" s="2" t="inlineStr"/>
+      <c r="M150" s="2" t="inlineStr">
+        <is>
+          <t>boltgatesuttoncoldfieldlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -7480,6 +7862,11 @@
       </c>
       <c r="K151" s="2" t="inlineStr"/>
       <c r="L151" s="2" t="inlineStr"/>
+      <c r="M151" s="2" t="inlineStr">
+        <is>
+          <t>keynestrugbylocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -7526,6 +7913,11 @@
       </c>
       <c r="K152" s="2" t="inlineStr"/>
       <c r="L152" s="2" t="inlineStr"/>
+      <c r="M152" s="2" t="inlineStr">
+        <is>
+          <t>keydashsolihulllocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -7572,6 +7964,11 @@
       </c>
       <c r="K153" s="2" t="inlineStr"/>
       <c r="L153" s="2" t="inlineStr"/>
+      <c r="M153" s="2" t="inlineStr">
+        <is>
+          <t>keyrisestaffordlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -7618,6 +8015,11 @@
       </c>
       <c r="K154" s="2" t="inlineStr"/>
       <c r="L154" s="2" t="inlineStr"/>
+      <c r="M154" s="2" t="inlineStr">
+        <is>
+          <t>latchrisewalsalllocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -7664,6 +8066,11 @@
       </c>
       <c r="K155" s="2" t="inlineStr"/>
       <c r="L155" s="2" t="inlineStr"/>
+      <c r="M155" s="2" t="inlineStr">
+        <is>
+          <t>locksprintwarwicklocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -7710,6 +8117,11 @@
       </c>
       <c r="K156" s="2" t="inlineStr"/>
       <c r="L156" s="2" t="inlineStr"/>
+      <c r="M156" s="2" t="inlineStr">
+        <is>
+          <t>lockzonewolverhamptonlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -7756,6 +8168,11 @@
       </c>
       <c r="K157" s="2" t="inlineStr"/>
       <c r="L157" s="2" t="inlineStr"/>
+      <c r="M157" s="2" t="inlineStr">
+        <is>
+          <t>boltdashworcesterlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -7802,6 +8219,11 @@
       </c>
       <c r="K158" s="2" t="inlineStr"/>
       <c r="L158" s="2" t="inlineStr"/>
+      <c r="M158" s="2" t="inlineStr">
+        <is>
+          <t>boltrisebarnsleylocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -7848,6 +8270,11 @@
       </c>
       <c r="K159" s="2" t="inlineStr"/>
       <c r="L159" s="2" t="inlineStr"/>
+      <c r="M159" s="2" t="inlineStr">
+        <is>
+          <t>lockquestharrogatelocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -7894,6 +8321,11 @@
       </c>
       <c r="K160" s="2" t="inlineStr"/>
       <c r="L160" s="2" t="inlineStr"/>
+      <c r="M160" s="2" t="inlineStr">
+        <is>
+          <t>boltstarhulllocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -7940,6 +8372,11 @@
       </c>
       <c r="K161" s="2" t="inlineStr"/>
       <c r="L161" s="2" t="inlineStr"/>
+      <c r="M161" s="2" t="inlineStr">
+        <is>
+          <t>keysquadmorleylocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -7986,6 +8423,11 @@
       </c>
       <c r="K162" s="2" t="inlineStr"/>
       <c r="L162" s="2" t="inlineStr"/>
+      <c r="M162" s="2" t="inlineStr">
+        <is>
+          <t>lockriserotherhamlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -8032,6 +8474,11 @@
       </c>
       <c r="K163" s="2" t="inlineStr"/>
       <c r="L163" s="2" t="inlineStr"/>
+      <c r="M163" s="2" t="inlineStr">
+        <is>
+          <t>lockedgewakefieldlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -8078,6 +8525,11 @@
       </c>
       <c r="K164" s="2" t="inlineStr"/>
       <c r="L164" s="2" t="inlineStr"/>
+      <c r="M164" s="2" t="inlineStr">
+        <is>
+          <t>latchlineyorklocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -8124,6 +8576,11 @@
         <v>1</v>
       </c>
       <c r="L165" s="2" t="inlineStr"/>
+      <c r="M165" s="2" t="inlineStr">
+        <is>
+          <t>ashington.doorfix-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
@@ -8170,6 +8627,11 @@
         <v>1</v>
       </c>
       <c r="L166" s="2" t="inlineStr"/>
+      <c r="M166" s="2" t="inlineStr">
+        <is>
+          <t>chester-le-street.doorfix-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
@@ -8216,6 +8678,11 @@
         <v>1</v>
       </c>
       <c r="L167" s="2" t="inlineStr"/>
+      <c r="M167" s="2" t="inlineStr">
+        <is>
+          <t>cramlington.doorfix-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -8262,6 +8729,11 @@
         <v>2</v>
       </c>
       <c r="L168" s="2" t="inlineStr"/>
+      <c r="M168" s="2" t="inlineStr">
+        <is>
+          <t>durham.keyfix-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -8308,6 +8780,11 @@
         <v>1</v>
       </c>
       <c r="L169" s="2" t="inlineStr"/>
+      <c r="M169" s="2" t="inlineStr">
+        <is>
+          <t>hebburn.doorfix-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
@@ -8354,6 +8831,11 @@
         <v>1</v>
       </c>
       <c r="L170" s="2" t="inlineStr"/>
+      <c r="M170" s="2" t="inlineStr">
+        <is>
+          <t>longbenton.doorfix-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -8400,6 +8882,11 @@
       </c>
       <c r="K171" s="2" t="inlineStr"/>
       <c r="L171" s="2" t="inlineStr"/>
+      <c r="M171" s="2" t="inlineStr">
+        <is>
+          <t>latchquestsouthshieldslocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
@@ -8446,6 +8933,11 @@
       </c>
       <c r="K172" s="2" t="inlineStr"/>
       <c r="L172" s="2" t="inlineStr"/>
+      <c r="M172" s="2" t="inlineStr">
+        <is>
+          <t>keysparktynemouthlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
@@ -8492,6 +8984,11 @@
         <v>1</v>
       </c>
       <c r="L173" s="2" t="inlineStr"/>
+      <c r="M173" s="2" t="inlineStr">
+        <is>
+          <t>wallsend.doorfix-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
@@ -8538,6 +9035,11 @@
         <v>1</v>
       </c>
       <c r="L174" s="2" t="inlineStr"/>
+      <c r="M174" s="2" t="inlineStr">
+        <is>
+          <t>whitley-bay.doorfix-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
@@ -8584,6 +9086,11 @@
         <v>2</v>
       </c>
       <c r="L175" s="2" t="inlineStr"/>
+      <c r="M175" s="2" t="inlineStr">
+        <is>
+          <t>billingham.keyfix-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
@@ -8630,6 +9137,11 @@
         <v>2</v>
       </c>
       <c r="L176" s="2" t="inlineStr"/>
+      <c r="M176" s="2" t="inlineStr">
+        <is>
+          <t>eston.keyfix-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
@@ -8676,6 +9188,11 @@
         <v>2</v>
       </c>
       <c r="L177" s="2" t="inlineStr"/>
+      <c r="M177" s="2" t="inlineStr">
+        <is>
+          <t>ingleby-barwick.keyfix-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
@@ -8722,6 +9239,11 @@
         <v>2</v>
       </c>
       <c r="L178" s="2" t="inlineStr"/>
+      <c r="M178" s="2" t="inlineStr">
+        <is>
+          <t>newton-aycliffe.keyfix-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
@@ -8768,6 +9290,11 @@
         <v>2</v>
       </c>
       <c r="L179" s="2" t="inlineStr"/>
+      <c r="M179" s="2" t="inlineStr">
+        <is>
+          <t>redcar.keyfix-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
@@ -8814,6 +9341,11 @@
         <v>2</v>
       </c>
       <c r="L180" s="2" t="inlineStr"/>
+      <c r="M180" s="2" t="inlineStr">
+        <is>
+          <t>thornaby-on-tees.keyfix-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
@@ -8860,6 +9392,11 @@
         <v>4</v>
       </c>
       <c r="L181" s="2" t="inlineStr"/>
+      <c r="M181" s="2" t="inlineStr">
+        <is>
+          <t>bingley.keypro-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
@@ -8906,6 +9443,11 @@
         <v>4</v>
       </c>
       <c r="L182" s="2" t="inlineStr"/>
+      <c r="M182" s="2" t="inlineStr">
+        <is>
+          <t>bramley.keypro-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
@@ -8952,6 +9494,11 @@
       </c>
       <c r="K183" s="2" t="inlineStr"/>
       <c r="L183" s="2" t="inlineStr"/>
+      <c r="M183" s="2" t="inlineStr">
+        <is>
+          <t>keyservedewsburylocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
@@ -8998,6 +9545,11 @@
         <v>4</v>
       </c>
       <c r="L184" s="2" t="inlineStr"/>
+      <c r="M184" s="2" t="inlineStr">
+        <is>
+          <t>keighley.keypro-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
@@ -9044,6 +9596,11 @@
         <v>3</v>
       </c>
       <c r="L185" s="2" t="inlineStr"/>
+      <c r="M185" s="2" t="inlineStr">
+        <is>
+          <t>accrington.keylok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
@@ -9090,6 +9647,11 @@
       </c>
       <c r="K186" s="2" t="inlineStr"/>
       <c r="L186" s="2" t="inlineStr"/>
+      <c r="M186" s="2" t="inlineStr">
+        <is>
+          <t>keymateblackburnlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
@@ -9136,6 +9698,11 @@
       </c>
       <c r="K187" s="2" t="inlineStr"/>
       <c r="L187" s="2" t="inlineStr"/>
+      <c r="M187" s="2" t="inlineStr">
+        <is>
+          <t>latchnodeburnleylocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
@@ -9182,6 +9749,11 @@
       </c>
       <c r="K188" s="2" t="inlineStr"/>
       <c r="L188" s="2" t="inlineStr"/>
+      <c r="M188" s="2" t="inlineStr">
+        <is>
+          <t>locknodeburylocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
@@ -9228,6 +9800,11 @@
         <v>3</v>
       </c>
       <c r="L189" s="2" t="inlineStr"/>
+      <c r="M189" s="2" t="inlineStr">
+        <is>
+          <t>darwen.keylok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
@@ -9274,6 +9851,11 @@
         <v>4</v>
       </c>
       <c r="L190" s="2" t="inlineStr"/>
+      <c r="M190" s="2" t="inlineStr">
+        <is>
+          <t>heywood.keypro-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
@@ -9320,6 +9902,11 @@
         <v>3</v>
       </c>
       <c r="L191" s="2" t="inlineStr"/>
+      <c r="M191" s="2" t="inlineStr">
+        <is>
+          <t>middleton.keylok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
@@ -9366,6 +9953,11 @@
         <v>3</v>
       </c>
       <c r="L192" s="2" t="inlineStr"/>
+      <c r="M192" s="2" t="inlineStr">
+        <is>
+          <t>nelson.keylok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
@@ -9412,6 +10004,11 @@
         <v>8</v>
       </c>
       <c r="L193" s="2" t="inlineStr"/>
+      <c r="M193" s="2" t="inlineStr">
+        <is>
+          <t>whitefield.ironlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
@@ -9458,6 +10055,11 @@
       </c>
       <c r="K194" s="2" t="inlineStr"/>
       <c r="L194" s="2" t="inlineStr"/>
+      <c r="M194" s="2" t="inlineStr">
+        <is>
+          <t>keyhavenhalifaxlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
@@ -9504,6 +10106,11 @@
         <v>6</v>
       </c>
       <c r="L195" s="2" t="inlineStr"/>
+      <c r="M195" s="2" t="inlineStr">
+        <is>
+          <t>ashton-in-makerfield.safelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
@@ -9550,6 +10157,11 @@
         <v>3</v>
       </c>
       <c r="L196" s="2" t="inlineStr"/>
+      <c r="M196" s="2" t="inlineStr">
+        <is>
+          <t>bamber-bridge.keylok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
@@ -9596,6 +10208,11 @@
         <v>3</v>
       </c>
       <c r="L197" s="2" t="inlineStr"/>
+      <c r="M197" s="2" t="inlineStr">
+        <is>
+          <t>fulwood.keylok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
@@ -9642,6 +10259,11 @@
         <v>6</v>
       </c>
       <c r="L198" s="2" t="inlineStr"/>
+      <c r="M198" s="2" t="inlineStr">
+        <is>
+          <t>hindley.safelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
@@ -9688,6 +10310,11 @@
         <v>3</v>
       </c>
       <c r="L199" s="2" t="inlineStr"/>
+      <c r="M199" s="2" t="inlineStr">
+        <is>
+          <t>leyland.keylok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
@@ -9734,6 +10361,11 @@
         <v>7</v>
       </c>
       <c r="L200" s="2" t="inlineStr"/>
+      <c r="M200" s="2" t="inlineStr">
+        <is>
+          <t>newton-le-willows.securelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
@@ -9780,6 +10412,11 @@
         <v>7</v>
       </c>
       <c r="L201" s="2" t="inlineStr"/>
+      <c r="M201" s="2" t="inlineStr">
+        <is>
+          <t>orrell.securelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
@@ -9826,6 +10463,11 @@
         <v>3</v>
       </c>
       <c r="L202" s="2" t="inlineStr"/>
+      <c r="M202" s="2" t="inlineStr">
+        <is>
+          <t>penwortham.keylok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
@@ -9872,6 +10514,11 @@
         <v>7</v>
       </c>
       <c r="L203" s="2" t="inlineStr"/>
+      <c r="M203" s="2" t="inlineStr">
+        <is>
+          <t>skelmersdale.securelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
@@ -9918,6 +10565,11 @@
       </c>
       <c r="K204" s="2" t="inlineStr"/>
       <c r="L204" s="2" t="inlineStr"/>
+      <c r="M204" s="2" t="inlineStr">
+        <is>
+          <t>latchcoresouthportlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
@@ -9964,6 +10616,11 @@
         <v>5</v>
       </c>
       <c r="L205" s="2" t="inlineStr"/>
+      <c r="M205" s="2" t="inlineStr">
+        <is>
+          <t>gainsborough.keysure-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
@@ -10010,6 +10667,11 @@
         <v>5</v>
       </c>
       <c r="L206" s="2" t="inlineStr"/>
+      <c r="M206" s="2" t="inlineStr">
+        <is>
+          <t>worksop.keysure-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
@@ -10056,6 +10718,11 @@
         <v>5</v>
       </c>
       <c r="L207" s="2" t="inlineStr"/>
+      <c r="M207" s="2" t="inlineStr">
+        <is>
+          <t>beverley.keysure-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
@@ -10102,6 +10769,11 @@
         <v>5</v>
       </c>
       <c r="L208" s="2" t="inlineStr"/>
+      <c r="M208" s="2" t="inlineStr">
+        <is>
+          <t>cleethorpes.keysure-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
@@ -10148,6 +10820,11 @@
         <v>5</v>
       </c>
       <c r="L209" s="2" t="inlineStr"/>
+      <c r="M209" s="2" t="inlineStr">
+        <is>
+          <t>goole.keysure-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
@@ -10194,6 +10871,11 @@
         <v>4</v>
       </c>
       <c r="L210" s="2" t="inlineStr"/>
+      <c r="M210" s="2" t="inlineStr">
+        <is>
+          <t>ossett.keypro-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
@@ -10240,6 +10922,11 @@
         <v>5</v>
       </c>
       <c r="L211" s="2" t="inlineStr"/>
+      <c r="M211" s="2" t="inlineStr">
+        <is>
+          <t>pontefract.keysure-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
@@ -10286,6 +10973,11 @@
         <v>5</v>
       </c>
       <c r="L212" s="2" t="inlineStr"/>
+      <c r="M212" s="2" t="inlineStr">
+        <is>
+          <t>rothwell.keysure-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
@@ -10332,6 +11024,11 @@
       </c>
       <c r="K213" s="2" t="inlineStr"/>
       <c r="L213" s="2" t="inlineStr"/>
+      <c r="M213" s="2" t="inlineStr">
+        <is>
+          <t>keynodescunthorpelocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
@@ -10378,6 +11075,11 @@
         <v>5</v>
       </c>
       <c r="L214" s="2" t="inlineStr"/>
+      <c r="M214" s="2" t="inlineStr">
+        <is>
+          <t>wickersley.keysure-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
@@ -10424,6 +11126,11 @@
         <v>8</v>
       </c>
       <c r="L215" s="2" t="inlineStr"/>
+      <c r="M215" s="2" t="inlineStr">
+        <is>
+          <t>ashton-under-lyne.ironlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
@@ -10470,6 +11177,11 @@
         <v>4</v>
       </c>
       <c r="L216" s="2" t="inlineStr"/>
+      <c r="M216" s="2" t="inlineStr">
+        <is>
+          <t>chadderton.keypro-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
@@ -10516,6 +11228,11 @@
         <v>8</v>
       </c>
       <c r="L217" s="2" t="inlineStr"/>
+      <c r="M217" s="2" t="inlineStr">
+        <is>
+          <t>denton.ironlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
@@ -10562,6 +11279,11 @@
         <v>8</v>
       </c>
       <c r="L218" s="2" t="inlineStr"/>
+      <c r="M218" s="2" t="inlineStr">
+        <is>
+          <t>droylsden.ironlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
@@ -10608,6 +11330,11 @@
         <v>4</v>
       </c>
       <c r="L219" s="2" t="inlineStr"/>
+      <c r="M219" s="2" t="inlineStr">
+        <is>
+          <t>dukinfield.keypro-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
@@ -10654,6 +11381,11 @@
         <v>8</v>
       </c>
       <c r="L220" s="2" t="inlineStr"/>
+      <c r="M220" s="2" t="inlineStr">
+        <is>
+          <t>hyde.ironlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
@@ -10700,6 +11432,11 @@
         <v>8</v>
       </c>
       <c r="L221" s="2" t="inlineStr"/>
+      <c r="M221" s="2" t="inlineStr">
+        <is>
+          <t>reddish.ironlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
@@ -10746,6 +11483,11 @@
         <v>4</v>
       </c>
       <c r="L222" s="2" t="inlineStr"/>
+      <c r="M222" s="2" t="inlineStr">
+        <is>
+          <t>royton.keypro-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
@@ -10792,6 +11534,11 @@
         <v>4</v>
       </c>
       <c r="L223" s="2" t="inlineStr"/>
+      <c r="M223" s="2" t="inlineStr">
+        <is>
+          <t>stalybridge.keypro-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
@@ -10838,6 +11585,11 @@
       </c>
       <c r="K224" s="2" t="inlineStr"/>
       <c r="L224" s="2" t="inlineStr"/>
+      <c r="M224" s="2" t="inlineStr">
+        <is>
+          <t>keylinkhuddersfieldlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
@@ -10884,6 +11636,11 @@
         <v>6</v>
       </c>
       <c r="L225" s="2" t="inlineStr"/>
+      <c r="M225" s="2" t="inlineStr">
+        <is>
+          <t>eccles.safelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
@@ -10930,6 +11687,11 @@
         <v>6</v>
       </c>
       <c r="L226" s="2" t="inlineStr"/>
+      <c r="M226" s="2" t="inlineStr">
+        <is>
+          <t>farnworth.safelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
@@ -10976,6 +11738,11 @@
         <v>6</v>
       </c>
       <c r="L227" s="2" t="inlineStr"/>
+      <c r="M227" s="2" t="inlineStr">
+        <is>
+          <t>golborne.safelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
@@ -11022,6 +11789,11 @@
         <v>6</v>
       </c>
       <c r="L228" s="2" t="inlineStr"/>
+      <c r="M228" s="2" t="inlineStr">
+        <is>
+          <t>leigh.safelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
@@ -11068,6 +11840,11 @@
         <v>6</v>
       </c>
       <c r="L229" s="2" t="inlineStr"/>
+      <c r="M229" s="2" t="inlineStr">
+        <is>
+          <t>little-hulton.safelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
@@ -11114,6 +11891,11 @@
         <v>8</v>
       </c>
       <c r="L230" s="2" t="inlineStr"/>
+      <c r="M230" s="2" t="inlineStr">
+        <is>
+          <t>old-trafford.ironlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
@@ -11160,6 +11942,11 @@
         <v>8</v>
       </c>
       <c r="L231" s="2" t="inlineStr"/>
+      <c r="M231" s="2" t="inlineStr">
+        <is>
+          <t>prestwich.ironlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
@@ -11206,6 +11993,11 @@
         <v>8</v>
       </c>
       <c r="L232" s="2" t="inlineStr"/>
+      <c r="M232" s="2" t="inlineStr">
+        <is>
+          <t>stretford.ironlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
@@ -11252,6 +12044,11 @@
         <v>6</v>
       </c>
       <c r="L233" s="2" t="inlineStr"/>
+      <c r="M233" s="2" t="inlineStr">
+        <is>
+          <t>swinton.safelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
@@ -11298,6 +12095,11 @@
         <v>6</v>
       </c>
       <c r="L234" s="2" t="inlineStr"/>
+      <c r="M234" s="2" t="inlineStr">
+        <is>
+          <t>urmston.safelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
@@ -11344,6 +12146,11 @@
       </c>
       <c r="K235" s="2" t="inlineStr"/>
       <c r="L235" s="2" t="inlineStr"/>
+      <c r="M235" s="2" t="inlineStr">
+        <is>
+          <t>keycraftbirkenheadlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
@@ -11390,6 +12197,11 @@
         <v>7</v>
       </c>
       <c r="L236" s="2" t="inlineStr"/>
+      <c r="M236" s="2" t="inlineStr">
+        <is>
+          <t>bootle.securelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
@@ -11436,6 +12248,11 @@
         <v>7</v>
       </c>
       <c r="L237" s="2" t="inlineStr"/>
+      <c r="M237" s="2" t="inlineStr">
+        <is>
+          <t>crosby.securelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
@@ -11482,6 +12299,11 @@
       </c>
       <c r="K238" s="2" t="inlineStr"/>
       <c r="L238" s="2" t="inlineStr"/>
+      <c r="M238" s="2" t="inlineStr">
+        <is>
+          <t>lockrouteellesmereportlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
@@ -11528,6 +12350,11 @@
         <v>7</v>
       </c>
       <c r="L239" s="2" t="inlineStr"/>
+      <c r="M239" s="2" t="inlineStr">
+        <is>
+          <t>formby.securelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
@@ -11574,6 +12401,11 @@
         <v>7</v>
       </c>
       <c r="L240" s="2" t="inlineStr"/>
+      <c r="M240" s="2" t="inlineStr">
+        <is>
+          <t>kirkby.securelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
@@ -11620,6 +12452,11 @@
         <v>7</v>
       </c>
       <c r="L241" s="2" t="inlineStr"/>
+      <c r="M241" s="2" t="inlineStr">
+        <is>
+          <t>maghull.securelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
@@ -11666,6 +12503,11 @@
         <v>7</v>
       </c>
       <c r="L242" s="2" t="inlineStr"/>
+      <c r="M242" s="2" t="inlineStr">
+        <is>
+          <t>prescot.securelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
@@ -11712,6 +12554,11 @@
       </c>
       <c r="K243" s="2" t="inlineStr"/>
       <c r="L243" s="2" t="inlineStr"/>
+      <c r="M243" s="2" t="inlineStr">
+        <is>
+          <t>lockdashsthelenslocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
@@ -11758,6 +12605,11 @@
         <v>9</v>
       </c>
       <c r="L244" s="2" t="inlineStr"/>
+      <c r="M244" s="2" t="inlineStr">
+        <is>
+          <t>widnes.steelfix-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
@@ -11804,6 +12656,11 @@
         <v>10</v>
       </c>
       <c r="L245" s="2" t="inlineStr"/>
+      <c r="M245" s="2" t="inlineStr">
+        <is>
+          <t>buxton.boltsafe-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
@@ -11850,6 +12707,11 @@
         <v>9</v>
       </c>
       <c r="L246" s="2" t="inlineStr"/>
+      <c r="M246" s="2" t="inlineStr">
+        <is>
+          <t>altrincham.steelfix-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
@@ -11896,6 +12758,11 @@
         <v>9</v>
       </c>
       <c r="L247" s="2" t="inlineStr"/>
+      <c r="M247" s="2" t="inlineStr">
+        <is>
+          <t>cheadle-hulme.steelfix-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
@@ -11942,6 +12809,11 @@
         <v>9</v>
       </c>
       <c r="L248" s="2" t="inlineStr"/>
+      <c r="M248" s="2" t="inlineStr">
+        <is>
+          <t>congleton.steelfix-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
@@ -11988,6 +12860,11 @@
       </c>
       <c r="K249" s="2" t="inlineStr"/>
       <c r="L249" s="2" t="inlineStr"/>
+      <c r="M249" s="2" t="inlineStr">
+        <is>
+          <t>boltquestcrewelocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
@@ -12034,6 +12911,11 @@
         <v>9</v>
       </c>
       <c r="L250" s="2" t="inlineStr"/>
+      <c r="M250" s="2" t="inlineStr">
+        <is>
+          <t>hazel-grove.steelfix-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
@@ -12080,6 +12962,11 @@
         <v>10</v>
       </c>
       <c r="L251" s="2" t="inlineStr"/>
+      <c r="M251" s="2" t="inlineStr">
+        <is>
+          <t>macclesfield.boltsafe-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
@@ -12126,6 +13013,11 @@
       </c>
       <c r="K252" s="2" t="inlineStr"/>
       <c r="L252" s="2" t="inlineStr"/>
+      <c r="M252" s="2" t="inlineStr">
+        <is>
+          <t>locksmartsalelocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
@@ -12172,6 +13064,11 @@
         <v>9</v>
       </c>
       <c r="L253" s="2" t="inlineStr"/>
+      <c r="M253" s="2" t="inlineStr">
+        <is>
+          <t>winsford.steelfix-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
@@ -12218,6 +13115,11 @@
       </c>
       <c r="K254" s="2" t="inlineStr"/>
       <c r="L254" s="2" t="inlineStr"/>
+      <c r="M254" s="2" t="inlineStr">
+        <is>
+          <t>boltedgewythenshawelocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
@@ -12264,6 +13166,11 @@
         <v>11</v>
       </c>
       <c r="L255" s="2" t="inlineStr"/>
+      <c r="M255" s="2" t="inlineStr">
+        <is>
+          <t>beeston.boltsure-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
@@ -12310,6 +13217,11 @@
         <v>14</v>
       </c>
       <c r="L256" s="2" t="inlineStr"/>
+      <c r="M256" s="2" t="inlineStr">
+        <is>
+          <t>carlton.durolok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
@@ -12356,6 +13268,11 @@
         <v>10</v>
       </c>
       <c r="L257" s="2" t="inlineStr"/>
+      <c r="M257" s="2" t="inlineStr">
+        <is>
+          <t>dronfield.boltsafe-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
@@ -12402,6 +13319,11 @@
         <v>11</v>
       </c>
       <c r="L258" s="2" t="inlineStr"/>
+      <c r="M258" s="2" t="inlineStr">
+        <is>
+          <t>heanor.boltsure-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
@@ -12448,6 +13370,11 @@
         <v>11</v>
       </c>
       <c r="L259" s="2" t="inlineStr"/>
+      <c r="M259" s="2" t="inlineStr">
+        <is>
+          <t>ilkeston.boltsure-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
@@ -12494,6 +13421,11 @@
         <v>10</v>
       </c>
       <c r="L260" s="2" t="inlineStr"/>
+      <c r="M260" s="2" t="inlineStr">
+        <is>
+          <t>kirkby-in-ashfield.boltsafe-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
@@ -12540,6 +13472,11 @@
         <v>11</v>
       </c>
       <c r="L261" s="2" t="inlineStr"/>
+      <c r="M261" s="2" t="inlineStr">
+        <is>
+          <t>long-eaton.boltsure-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
@@ -12586,6 +13523,11 @@
       </c>
       <c r="K262" s="2" t="inlineStr"/>
       <c r="L262" s="2" t="inlineStr"/>
+      <c r="M262" s="2" t="inlineStr">
+        <is>
+          <t>lockservemansfieldlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
@@ -12632,6 +13574,11 @@
         <v>10</v>
       </c>
       <c r="L263" s="2" t="inlineStr"/>
+      <c r="M263" s="2" t="inlineStr">
+        <is>
+          <t>ripley.boltsafe-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
@@ -12678,6 +13625,11 @@
         <v>10</v>
       </c>
       <c r="L264" s="2" t="inlineStr"/>
+      <c r="M264" s="2" t="inlineStr">
+        <is>
+          <t>sutton-in-ashfield.boltsafe-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
@@ -12724,6 +13676,11 @@
         <v>11</v>
       </c>
       <c r="L265" s="2" t="inlineStr"/>
+      <c r="M265" s="2" t="inlineStr">
+        <is>
+          <t>clifton.boltsure-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
@@ -12770,6 +13727,11 @@
         <v>11</v>
       </c>
       <c r="L266" s="2" t="inlineStr"/>
+      <c r="M266" s="2" t="inlineStr">
+        <is>
+          <t>coalville.boltsure-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
@@ -12816,6 +13778,11 @@
       </c>
       <c r="K267" s="2" t="inlineStr"/>
       <c r="L267" s="2" t="inlineStr"/>
+      <c r="M267" s="2" t="inlineStr">
+        <is>
+          <t>boltrootcorbylocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
@@ -12862,6 +13829,11 @@
         <v>12</v>
       </c>
       <c r="L268" s="2" t="inlineStr"/>
+      <c r="M268" s="2" t="inlineStr">
+        <is>
+          <t>grantham.latchfix-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
@@ -12908,6 +13880,11 @@
         <v>12</v>
       </c>
       <c r="L269" s="2" t="inlineStr"/>
+      <c r="M269" s="2" t="inlineStr">
+        <is>
+          <t>market-harborough.latchfix-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
@@ -12954,6 +13931,11 @@
         <v>12</v>
       </c>
       <c r="L270" s="2" t="inlineStr"/>
+      <c r="M270" s="2" t="inlineStr">
+        <is>
+          <t>melton-mowbray.latchfix-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
@@ -13000,6 +13982,11 @@
         <v>12</v>
       </c>
       <c r="L271" s="2" t="inlineStr"/>
+      <c r="M271" s="2" t="inlineStr">
+        <is>
+          <t>oadby.latchfix-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
@@ -13046,6 +14033,11 @@
         <v>12</v>
       </c>
       <c r="L272" s="2" t="inlineStr"/>
+      <c r="M272" s="2" t="inlineStr">
+        <is>
+          <t>spalding.latchfix-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
@@ -13092,6 +14084,11 @@
         <v>12</v>
       </c>
       <c r="L273" s="2" t="inlineStr"/>
+      <c r="M273" s="2" t="inlineStr">
+        <is>
+          <t>stamford.latchfix-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
@@ -13138,6 +14135,11 @@
         <v>12</v>
       </c>
       <c r="L274" s="2" t="inlineStr"/>
+      <c r="M274" s="2" t="inlineStr">
+        <is>
+          <t>wigston.latchfix-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" s="2" t="inlineStr">
@@ -13184,6 +14186,11 @@
         <v>14</v>
       </c>
       <c r="L275" s="2" t="inlineStr"/>
+      <c r="M275" s="2" t="inlineStr">
+        <is>
+          <t>hinckley.durolok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" s="2" t="inlineStr">
@@ -13230,6 +14237,11 @@
         <v>11</v>
       </c>
       <c r="L276" s="2" t="inlineStr"/>
+      <c r="M276" s="2" t="inlineStr">
+        <is>
+          <t>swadlincote.boltsure-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
@@ -13276,6 +14288,11 @@
         <v>14</v>
       </c>
       <c r="L277" s="2" t="inlineStr"/>
+      <c r="M277" s="2" t="inlineStr">
+        <is>
+          <t>bedworth.durolok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
@@ -13322,6 +14339,11 @@
         <v>9</v>
       </c>
       <c r="L278" s="2" t="inlineStr"/>
+      <c r="M278" s="2" t="inlineStr">
+        <is>
+          <t>brownhills.steelfix-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
@@ -13368,6 +14390,11 @@
       </c>
       <c r="K279" s="2" t="inlineStr"/>
       <c r="L279" s="2" t="inlineStr"/>
+      <c r="M279" s="2" t="inlineStr">
+        <is>
+          <t>keysmartcannocklocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
@@ -13414,6 +14441,11 @@
       </c>
       <c r="K280" s="2" t="inlineStr"/>
       <c r="L280" s="2" t="inlineStr"/>
+      <c r="M280" s="2" t="inlineStr">
+        <is>
+          <t>latchgridnuneatonlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
@@ -13460,6 +14492,11 @@
         <v>10</v>
       </c>
       <c r="L281" s="2" t="inlineStr"/>
+      <c r="M281" s="2" t="inlineStr">
+        <is>
+          <t>rugeley.boltsafe-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
@@ -13506,6 +14543,11 @@
         <v>14</v>
       </c>
       <c r="L282" s="2" t="inlineStr"/>
+      <c r="M282" s="2" t="inlineStr">
+        <is>
+          <t>smethwick.durolok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
@@ -13552,6 +14594,11 @@
         <v>13</v>
       </c>
       <c r="L283" s="2" t="inlineStr"/>
+      <c r="M283" s="2" t="inlineStr">
+        <is>
+          <t>wednesbury.latchlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" s="2" t="inlineStr">
@@ -13598,6 +14645,11 @@
       </c>
       <c r="K284" s="2" t="inlineStr"/>
       <c r="L284" s="2" t="inlineStr"/>
+      <c r="M284" s="2" t="inlineStr">
+        <is>
+          <t>latchdashwestbromwichlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
@@ -13644,6 +14696,11 @@
         <v>13</v>
       </c>
       <c r="L285" s="2" t="inlineStr"/>
+      <c r="M285" s="2" t="inlineStr">
+        <is>
+          <t>bilston.latchlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
@@ -13690,6 +14747,11 @@
         <v>13</v>
       </c>
       <c r="L286" s="2" t="inlineStr"/>
+      <c r="M286" s="2" t="inlineStr">
+        <is>
+          <t>brierley-hill.latchlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" s="2" t="inlineStr">
@@ -13736,6 +14798,11 @@
         <v>13</v>
       </c>
       <c r="L287" s="2" t="inlineStr"/>
+      <c r="M287" s="2" t="inlineStr">
+        <is>
+          <t>kingswinford.latchlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" s="2" t="inlineStr">
@@ -13782,6 +14849,11 @@
         <v>14</v>
       </c>
       <c r="L288" s="2" t="inlineStr"/>
+      <c r="M288" s="2" t="inlineStr">
+        <is>
+          <t>oldbury.durolok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" s="2" t="inlineStr">
@@ -13828,6 +14900,11 @@
         <v>14</v>
       </c>
       <c r="L289" s="2" t="inlineStr"/>
+      <c r="M289" s="2" t="inlineStr">
+        <is>
+          <t>rowley-regis.durolok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
@@ -13874,6 +14951,11 @@
         <v>13</v>
       </c>
       <c r="L290" s="2" t="inlineStr"/>
+      <c r="M290" s="2" t="inlineStr">
+        <is>
+          <t>sedgley.latchlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" s="2" t="inlineStr">
@@ -13920,6 +15002,11 @@
         <v>15</v>
       </c>
       <c r="L291" s="2" t="inlineStr"/>
+      <c r="M291" s="2" t="inlineStr">
+        <is>
+          <t>stourbridge.primelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" s="2" t="inlineStr">
@@ -13966,6 +15053,11 @@
       </c>
       <c r="K292" s="2" t="inlineStr"/>
       <c r="L292" s="2" t="inlineStr"/>
+      <c r="M292" s="2" t="inlineStr">
+        <is>
+          <t>latchpointtelfordlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" s="2" t="inlineStr">
@@ -14012,6 +15104,11 @@
         <v>13</v>
       </c>
       <c r="L293" s="2" t="inlineStr"/>
+      <c r="M293" s="2" t="inlineStr">
+        <is>
+          <t>tipton.latchlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
@@ -14058,6 +15155,11 @@
         <v>13</v>
       </c>
       <c r="L294" s="2" t="inlineStr"/>
+      <c r="M294" s="2" t="inlineStr">
+        <is>
+          <t>willenhall.latchlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
@@ -14104,6 +15206,11 @@
       </c>
       <c r="K295" s="2" t="inlineStr"/>
       <c r="L295" s="2" t="inlineStr"/>
+      <c r="M295" s="2" t="inlineStr">
+        <is>
+          <t>latchserveketteringlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
@@ -14150,6 +15257,11 @@
         <v>16</v>
       </c>
       <c r="L296" s="2" t="inlineStr"/>
+      <c r="M296" s="2" t="inlineStr">
+        <is>
+          <t>rushden.truebolt-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
@@ -14196,6 +15308,11 @@
         <v>16</v>
       </c>
       <c r="L297" s="2" t="inlineStr"/>
+      <c r="M297" s="2" t="inlineStr">
+        <is>
+          <t>wellingborough.truebolt-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" s="2" t="inlineStr">
@@ -14242,6 +15359,11 @@
         <v>16</v>
       </c>
       <c r="L298" s="2" t="inlineStr"/>
+      <c r="M298" s="2" t="inlineStr">
+        <is>
+          <t>biggleswade.truebolt-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
@@ -14288,6 +15410,11 @@
         <v>17</v>
       </c>
       <c r="L299" s="2" t="inlineStr"/>
+      <c r="M299" s="2" t="inlineStr">
+        <is>
+          <t>bury-st-edmunds.surebolt-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
@@ -14334,6 +15461,11 @@
         <v>16</v>
       </c>
       <c r="L300" s="2" t="inlineStr"/>
+      <c r="M300" s="2" t="inlineStr">
+        <is>
+          <t>kempston.truebolt-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
@@ -14380,6 +15512,11 @@
         <v>16</v>
       </c>
       <c r="L301" s="2" t="inlineStr"/>
+      <c r="M301" s="2" t="inlineStr">
+        <is>
+          <t>letchworth.truebolt-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="302">
       <c r="A302" s="2" t="inlineStr">
@@ -14426,6 +15563,11 @@
         <v>16</v>
       </c>
       <c r="L302" s="2" t="inlineStr"/>
+      <c r="M302" s="2" t="inlineStr">
+        <is>
+          <t>st-neots.truebolt-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="303">
       <c r="A303" s="2" t="inlineStr">
@@ -14472,6 +15614,11 @@
         <v>17</v>
       </c>
       <c r="L303" s="2" t="inlineStr"/>
+      <c r="M303" s="2" t="inlineStr">
+        <is>
+          <t>sudbury.surebolt-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="304">
       <c r="A304" s="2" t="inlineStr">
@@ -14518,6 +15665,11 @@
         <v>12</v>
       </c>
       <c r="L304" s="2" t="inlineStr"/>
+      <c r="M304" s="2" t="inlineStr">
+        <is>
+          <t>wisbech.latchfix-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" s="2" t="inlineStr">
@@ -14564,6 +15716,11 @@
         <v>18</v>
       </c>
       <c r="L305" s="2" t="inlineStr"/>
+      <c r="M305" s="2" t="inlineStr">
+        <is>
+          <t>banbury.boltright-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="306">
       <c r="A306" s="2" t="inlineStr">
@@ -14610,6 +15767,11 @@
         <v>18</v>
       </c>
       <c r="L306" s="2" t="inlineStr"/>
+      <c r="M306" s="2" t="inlineStr">
+        <is>
+          <t>bicester.boltright-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
@@ -14656,6 +15818,11 @@
         <v>15</v>
       </c>
       <c r="L307" s="2" t="inlineStr"/>
+      <c r="M307" s="2" t="inlineStr">
+        <is>
+          <t>quedgeley-and-hardwicke.primelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="308">
       <c r="A308" s="2" t="inlineStr">
@@ -14702,6 +15869,11 @@
         <v>15</v>
       </c>
       <c r="L308" s="2" t="inlineStr"/>
+      <c r="M308" s="2" t="inlineStr">
+        <is>
+          <t>droitwich-spa.primelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="309">
       <c r="A309" s="2" t="inlineStr">
@@ -14748,6 +15920,11 @@
         <v>15</v>
       </c>
       <c r="L309" s="2" t="inlineStr"/>
+      <c r="M309" s="2" t="inlineStr">
+        <is>
+          <t>evesham.primelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
@@ -14794,6 +15971,11 @@
       </c>
       <c r="K310" s="2" t="inlineStr"/>
       <c r="L310" s="2" t="inlineStr"/>
+      <c r="M310" s="2" t="inlineStr">
+        <is>
+          <t>locksparkhalesowenlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="311">
       <c r="A311" s="2" t="inlineStr">
@@ -14840,6 +16022,11 @@
         <v>14</v>
       </c>
       <c r="L311" s="2" t="inlineStr"/>
+      <c r="M311" s="2" t="inlineStr">
+        <is>
+          <t>kenilworth.durolok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="312">
       <c r="A312" s="2" t="inlineStr">
@@ -14886,6 +16073,11 @@
         <v>15</v>
       </c>
       <c r="L312" s="2" t="inlineStr"/>
+      <c r="M312" s="2" t="inlineStr">
+        <is>
+          <t>kidderminster.primelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="313">
       <c r="A313" s="2" t="inlineStr">
@@ -14932,6 +16124,11 @@
         <v>15</v>
       </c>
       <c r="L313" s="2" t="inlineStr"/>
+      <c r="M313" s="2" t="inlineStr">
+        <is>
+          <t>stourport-on-severn.primelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="314">
       <c r="A314" s="2" t="inlineStr">
@@ -14978,6 +16175,11 @@
         <v>15</v>
       </c>
       <c r="L314" s="2" t="inlineStr"/>
+      <c r="M314" s="2" t="inlineStr">
+        <is>
+          <t>stratford-upon-avon.primelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" s="2" t="inlineStr">
@@ -15024,6 +16226,11 @@
         <v>20</v>
       </c>
       <c r="L315" s="2" t="inlineStr"/>
+      <c r="M315" s="2" t="inlineStr">
+        <is>
+          <t>berkhamsted.guardlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="316">
       <c r="A316" s="2" t="inlineStr">
@@ -15070,6 +16277,11 @@
         <v>20</v>
       </c>
       <c r="L316" s="2" t="inlineStr"/>
+      <c r="M316" s="2" t="inlineStr">
+        <is>
+          <t>bushey.guardlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="317">
       <c r="A317" s="2" t="inlineStr">
@@ -15116,6 +16328,11 @@
         <v>16</v>
       </c>
       <c r="L317" s="2" t="inlineStr"/>
+      <c r="M317" s="2" t="inlineStr">
+        <is>
+          <t>dunstable.truebolt-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="318">
       <c r="A318" s="2" t="inlineStr">
@@ -15162,6 +16379,11 @@
         <v>16</v>
       </c>
       <c r="L318" s="2" t="inlineStr"/>
+      <c r="M318" s="2" t="inlineStr">
+        <is>
+          <t>harpenden.truebolt-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" s="2" t="inlineStr">
@@ -15208,6 +16430,11 @@
         <v>16</v>
       </c>
       <c r="L319" s="2" t="inlineStr"/>
+      <c r="M319" s="2" t="inlineStr">
+        <is>
+          <t>hitchin.truebolt-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
@@ -15254,6 +16481,11 @@
         <v>18</v>
       </c>
       <c r="L320" s="2" t="inlineStr"/>
+      <c r="M320" s="2" t="inlineStr">
+        <is>
+          <t>leighton-buzzard.boltright-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="321">
       <c r="A321" s="2" t="inlineStr">
@@ -15300,6 +16532,11 @@
         <v>20</v>
       </c>
       <c r="L321" s="2" t="inlineStr"/>
+      <c r="M321" s="2" t="inlineStr">
+        <is>
+          <t>rickmansworth.guardlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="322">
       <c r="A322" s="2" t="inlineStr">
@@ -15346,6 +16583,11 @@
       </c>
       <c r="K322" s="2" t="inlineStr"/>
       <c r="L322" s="2" t="inlineStr"/>
+      <c r="M322" s="2" t="inlineStr">
+        <is>
+          <t>boltlinkwatfordlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="323">
       <c r="A323" s="2" t="inlineStr">
@@ -15392,6 +16634,11 @@
         <v>18</v>
       </c>
       <c r="L323" s="2" t="inlineStr"/>
+      <c r="M323" s="2" t="inlineStr">
+        <is>
+          <t>bletchley.boltright-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="324">
       <c r="A324" s="2" t="inlineStr">
@@ -15438,6 +16685,11 @@
         <v>20</v>
       </c>
       <c r="L324" s="2" t="inlineStr"/>
+      <c r="M324" s="2" t="inlineStr">
+        <is>
+          <t>hazlemere.guardlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="325">
       <c r="A325" s="2" t="inlineStr">
@@ -15484,6 +16736,11 @@
         <v>19</v>
       </c>
       <c r="L325" s="2" t="inlineStr"/>
+      <c r="M325" s="2" t="inlineStr">
+        <is>
+          <t>billericay.gatelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="326">
       <c r="A326" s="2" t="inlineStr">
@@ -15530,6 +16787,11 @@
         <v>19</v>
       </c>
       <c r="L326" s="2" t="inlineStr"/>
+      <c r="M326" s="2" t="inlineStr">
+        <is>
+          <t>bishop-s-stortford.gatelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="327">
       <c r="A327" s="2" t="inlineStr">
@@ -15576,6 +16838,11 @@
         <v>19</v>
       </c>
       <c r="L327" s="2" t="inlineStr"/>
+      <c r="M327" s="2" t="inlineStr">
+        <is>
+          <t>brentwood.gatelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="328">
       <c r="A328" s="2" t="inlineStr">
@@ -15622,6 +16889,11 @@
         <v>19</v>
       </c>
       <c r="L328" s="2" t="inlineStr"/>
+      <c r="M328" s="2" t="inlineStr">
+        <is>
+          <t>cheshunt.gatelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="329">
       <c r="A329" s="2" t="inlineStr">
@@ -15668,6 +16940,11 @@
         <v>19</v>
       </c>
       <c r="L329" s="2" t="inlineStr"/>
+      <c r="M329" s="2" t="inlineStr">
+        <is>
+          <t>hatfield.gatelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="330">
       <c r="A330" s="2" t="inlineStr">
@@ -15714,6 +16991,11 @@
         <v>19</v>
       </c>
       <c r="L330" s="2" t="inlineStr"/>
+      <c r="M330" s="2" t="inlineStr">
+        <is>
+          <t>hertford.gatelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="331">
       <c r="A331" s="2" t="inlineStr">
@@ -15760,6 +17042,11 @@
         <v>19</v>
       </c>
       <c r="L331" s="2" t="inlineStr"/>
+      <c r="M331" s="2" t="inlineStr">
+        <is>
+          <t>hoddesdon.gatelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="332">
       <c r="A332" s="2" t="inlineStr">
@@ -15806,6 +17093,11 @@
         <v>19</v>
       </c>
       <c r="L332" s="2" t="inlineStr"/>
+      <c r="M332" s="2" t="inlineStr">
+        <is>
+          <t>loughton.gatelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="333">
       <c r="A333" s="2" t="inlineStr">
@@ -15852,6 +17144,11 @@
         <v>19</v>
       </c>
       <c r="L333" s="2" t="inlineStr"/>
+      <c r="M333" s="2" t="inlineStr">
+        <is>
+          <t>potters-bar.gatelok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="334">
       <c r="A334" s="2" t="inlineStr">
@@ -15898,6 +17195,11 @@
         <v>17</v>
       </c>
       <c r="L334" s="2" t="inlineStr"/>
+      <c r="M334" s="2" t="inlineStr">
+        <is>
+          <t>wickford.surebolt-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="335">
       <c r="A335" s="2" t="inlineStr">
@@ -15944,6 +17246,11 @@
         <v>17</v>
       </c>
       <c r="L335" s="2" t="inlineStr"/>
+      <c r="M335" s="2" t="inlineStr">
+        <is>
+          <t>clacton-on-sea.surebolt-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="336">
       <c r="A336" s="2" t="inlineStr">
@@ -15990,6 +17297,11 @@
         <v>17</v>
       </c>
       <c r="L336" s="2" t="inlineStr"/>
+      <c r="M336" s="2" t="inlineStr">
+        <is>
+          <t>felixstowe.surebolt-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="337">
       <c r="A337" s="2" t="inlineStr">
@@ -16036,6 +17348,11 @@
         <v>17</v>
       </c>
       <c r="L337" s="2" t="inlineStr"/>
+      <c r="M337" s="2" t="inlineStr">
+        <is>
+          <t>harwich.surebolt-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
@@ -16082,6 +17399,11 @@
         <v>17</v>
       </c>
       <c r="L338" s="2" t="inlineStr"/>
+      <c r="M338" s="2" t="inlineStr">
+        <is>
+          <t>maldon.surebolt-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" s="2" t="inlineStr">
@@ -16128,6 +17450,11 @@
         <v>17</v>
       </c>
       <c r="L339" s="2" t="inlineStr"/>
+      <c r="M339" s="2" t="inlineStr">
+        <is>
+          <t>rayleigh.surebolt-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="340">
       <c r="A340" s="2" t="inlineStr">
@@ -16174,6 +17501,11 @@
         <v>17</v>
       </c>
       <c r="L340" s="2" t="inlineStr"/>
+      <c r="M340" s="2" t="inlineStr">
+        <is>
+          <t>witham.surebolt-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="341">
       <c r="A341" s="2" t="inlineStr">
@@ -16220,6 +17552,11 @@
         <v>22</v>
       </c>
       <c r="L341" s="2" t="inlineStr"/>
+      <c r="M341" s="2" t="inlineStr">
+        <is>
+          <t>broadstairs.keyguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="342">
       <c r="A342" s="2" t="inlineStr">
@@ -16266,6 +17603,11 @@
       </c>
       <c r="K342" s="2" t="inlineStr"/>
       <c r="L342" s="2" t="inlineStr"/>
+      <c r="M342" s="2" t="inlineStr">
+        <is>
+          <t>boltservemargatelocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="343">
       <c r="A343" s="2" t="inlineStr">
@@ -16312,6 +17654,11 @@
         <v>22</v>
       </c>
       <c r="L343" s="2" t="inlineStr"/>
+      <c r="M343" s="2" t="inlineStr">
+        <is>
+          <t>ramsgate.keyguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="344">
       <c r="A344" s="2" t="inlineStr">
@@ -16358,6 +17705,11 @@
         <v>22</v>
       </c>
       <c r="L344" s="2" t="inlineStr"/>
+      <c r="M344" s="2" t="inlineStr">
+        <is>
+          <t>whitstable.keyguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="345">
       <c r="A345" s="2" t="inlineStr">
@@ -16404,6 +17756,11 @@
       </c>
       <c r="K345" s="2" t="inlineStr"/>
       <c r="L345" s="2" t="inlineStr"/>
+      <c r="M345" s="2" t="inlineStr">
+        <is>
+          <t>keymaxbasingstokelocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
@@ -16450,6 +17807,11 @@
         <v>18</v>
       </c>
       <c r="L346" s="2" t="inlineStr"/>
+      <c r="M346" s="2" t="inlineStr">
+        <is>
+          <t>didcot.boltright-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="347">
       <c r="A347" s="2" t="inlineStr">
@@ -16496,6 +17858,11 @@
         <v>25</v>
       </c>
       <c r="L347" s="2" t="inlineStr"/>
+      <c r="M347" s="2" t="inlineStr">
+        <is>
+          <t>fleet.sureguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="348">
       <c r="A348" s="2" t="inlineStr">
@@ -16542,6 +17909,11 @@
       </c>
       <c r="K348" s="2" t="inlineStr"/>
       <c r="L348" s="2" t="inlineStr"/>
+      <c r="M348" s="2" t="inlineStr">
+        <is>
+          <t>keykinghighwycombelocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" s="2" t="inlineStr">
@@ -16588,6 +17960,11 @@
         <v>18</v>
       </c>
       <c r="L349" s="2" t="inlineStr"/>
+      <c r="M349" s="2" t="inlineStr">
+        <is>
+          <t>newbury.boltright-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="350">
       <c r="A350" s="2" t="inlineStr">
@@ -16634,6 +18011,11 @@
         <v>25</v>
       </c>
       <c r="L350" s="2" t="inlineStr"/>
+      <c r="M350" s="2" t="inlineStr">
+        <is>
+          <t>sandhurst.sureguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="351">
       <c r="A351" s="2" t="inlineStr">
@@ -16680,6 +18062,11 @@
         <v>18</v>
       </c>
       <c r="L351" s="2" t="inlineStr"/>
+      <c r="M351" s="2" t="inlineStr">
+        <is>
+          <t>thatcham.boltright-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="352">
       <c r="A352" s="2" t="inlineStr">
@@ -16726,6 +18113,11 @@
         <v>25</v>
       </c>
       <c r="L352" s="2" t="inlineStr"/>
+      <c r="M352" s="2" t="inlineStr">
+        <is>
+          <t>woodley.sureguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="353">
       <c r="A353" s="2" t="inlineStr">
@@ -16772,6 +18164,11 @@
       </c>
       <c r="K353" s="2" t="inlineStr"/>
       <c r="L353" s="2" t="inlineStr"/>
+      <c r="M353" s="2" t="inlineStr">
+        <is>
+          <t>keypeakswindonlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="354">
       <c r="A354" s="2" t="inlineStr">
@@ -16818,6 +18215,11 @@
         <v>22</v>
       </c>
       <c r="L354" s="2" t="inlineStr"/>
+      <c r="M354" s="2" t="inlineStr">
+        <is>
+          <t>canvey-island.keyguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="355">
       <c r="A355" s="2" t="inlineStr">
@@ -16864,6 +18266,11 @@
         <v>22</v>
       </c>
       <c r="L355" s="2" t="inlineStr"/>
+      <c r="M355" s="2" t="inlineStr">
+        <is>
+          <t>south-benfleet.keyguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="356">
       <c r="A356" s="2" t="inlineStr">
@@ -16910,6 +18317,11 @@
         <v>24</v>
       </c>
       <c r="L356" s="2" t="inlineStr"/>
+      <c r="M356" s="2" t="inlineStr">
+        <is>
+          <t>south-ockendon.boltguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="357">
       <c r="A357" s="2" t="inlineStr">
@@ -16956,6 +18368,11 @@
       </c>
       <c r="K357" s="2" t="inlineStr"/>
       <c r="L357" s="2" t="inlineStr"/>
+      <c r="M357" s="2" t="inlineStr">
+        <is>
+          <t>boltnestchathamlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
@@ -17002,6 +18419,11 @@
       </c>
       <c r="K358" s="2" t="inlineStr"/>
       <c r="L358" s="2" t="inlineStr"/>
+      <c r="M358" s="2" t="inlineStr">
+        <is>
+          <t>keyrootdartfordlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="359">
       <c r="A359" s="2" t="inlineStr">
@@ -17048,6 +18470,11 @@
         <v>24</v>
       </c>
       <c r="L359" s="2" t="inlineStr"/>
+      <c r="M359" s="2" t="inlineStr">
+        <is>
+          <t>larkfield.boltguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
@@ -17094,6 +18521,11 @@
         <v>24</v>
       </c>
       <c r="L360" s="2" t="inlineStr"/>
+      <c r="M360" s="2" t="inlineStr">
+        <is>
+          <t>northfleet.boltguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="361">
       <c r="A361" s="2" t="inlineStr">
@@ -17140,6 +18572,11 @@
       </c>
       <c r="K361" s="2" t="inlineStr"/>
       <c r="L361" s="2" t="inlineStr"/>
+      <c r="M361" s="2" t="inlineStr">
+        <is>
+          <t>keyrouterochesterlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="362">
       <c r="A362" s="2" t="inlineStr">
@@ -17186,6 +18623,11 @@
         <v>24</v>
       </c>
       <c r="L362" s="2" t="inlineStr"/>
+      <c r="M362" s="2" t="inlineStr">
+        <is>
+          <t>sevenoaks.boltguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="363">
       <c r="A363" s="2" t="inlineStr">
@@ -17232,6 +18674,11 @@
         <v>20</v>
       </c>
       <c r="L363" s="2" t="inlineStr"/>
+      <c r="M363" s="2" t="inlineStr">
+        <is>
+          <t>ascot.guardlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="364">
       <c r="A364" s="2" t="inlineStr">
@@ -17278,6 +18725,11 @@
         <v>25</v>
       </c>
       <c r="L364" s="2" t="inlineStr"/>
+      <c r="M364" s="2" t="inlineStr">
+        <is>
+          <t>ash-and-ash-vale.sureguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="365">
       <c r="A365" s="2" t="inlineStr">
@@ -17324,6 +18776,11 @@
       </c>
       <c r="K365" s="2" t="inlineStr"/>
       <c r="L365" s="2" t="inlineStr"/>
+      <c r="M365" s="2" t="inlineStr">
+        <is>
+          <t>boltnodebracknelllocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="366">
       <c r="A366" s="2" t="inlineStr">
@@ -17370,6 +18827,11 @@
         <v>20</v>
       </c>
       <c r="L366" s="2" t="inlineStr"/>
+      <c r="M366" s="2" t="inlineStr">
+        <is>
+          <t>camberley.guardlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="367">
       <c r="A367" s="2" t="inlineStr">
@@ -17416,6 +18878,11 @@
         <v>20</v>
       </c>
       <c r="L367" s="2" t="inlineStr"/>
+      <c r="M367" s="2" t="inlineStr">
+        <is>
+          <t>egham.guardlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
@@ -17462,6 +18929,11 @@
       </c>
       <c r="K368" s="2" t="inlineStr"/>
       <c r="L368" s="2" t="inlineStr"/>
+      <c r="M368" s="2" t="inlineStr">
+        <is>
+          <t>latchrootmaidenheadlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="369">
       <c r="A369" s="2" t="inlineStr">
@@ -17508,6 +18980,11 @@
         <v>23</v>
       </c>
       <c r="L369" s="2" t="inlineStr"/>
+      <c r="M369" s="2" t="inlineStr">
+        <is>
+          <t>sheerwater.lockguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="370">
       <c r="A370" s="2" t="inlineStr">
@@ -17554,6 +19031,11 @@
         <v>20</v>
       </c>
       <c r="L370" s="2" t="inlineStr"/>
+      <c r="M370" s="2" t="inlineStr">
+        <is>
+          <t>staines-upon-thames.guardlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="371">
       <c r="A371" s="2" t="inlineStr">
@@ -17600,6 +19082,11 @@
         <v>23</v>
       </c>
       <c r="L371" s="2" t="inlineStr"/>
+      <c r="M371" s="2" t="inlineStr">
+        <is>
+          <t>west-byfleet.lockguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="372">
       <c r="A372" s="2" t="inlineStr">
@@ -17646,6 +19133,11 @@
         <v>20</v>
       </c>
       <c r="L372" s="2" t="inlineStr"/>
+      <c r="M372" s="2" t="inlineStr">
+        <is>
+          <t>windsor.guardlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="373">
       <c r="A373" s="2" t="inlineStr">
@@ -17692,6 +19184,11 @@
         <v>23</v>
       </c>
       <c r="L373" s="2" t="inlineStr"/>
+      <c r="M373" s="2" t="inlineStr">
+        <is>
+          <t>epsom.lockguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="374">
       <c r="A374" s="2" t="inlineStr">
@@ -17738,6 +19235,11 @@
         <v>23</v>
       </c>
       <c r="L374" s="2" t="inlineStr"/>
+      <c r="M374" s="2" t="inlineStr">
+        <is>
+          <t>epsom-downs.lockguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="375">
       <c r="A375" s="2" t="inlineStr">
@@ -17784,6 +19286,11 @@
         <v>23</v>
       </c>
       <c r="L375" s="2" t="inlineStr"/>
+      <c r="M375" s="2" t="inlineStr">
+        <is>
+          <t>ewell.lockguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="376">
       <c r="A376" s="2" t="inlineStr">
@@ -17830,6 +19337,11 @@
         <v>23</v>
       </c>
       <c r="L376" s="2" t="inlineStr"/>
+      <c r="M376" s="2" t="inlineStr">
+        <is>
+          <t>new-haw.lockguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="377">
       <c r="A377" s="2" t="inlineStr">
@@ -17876,6 +19388,11 @@
         <v>24</v>
       </c>
       <c r="L377" s="2" t="inlineStr"/>
+      <c r="M377" s="2" t="inlineStr">
+        <is>
+          <t>redhill.boltguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="378">
       <c r="A378" s="2" t="inlineStr">
@@ -17922,6 +19439,11 @@
         <v>24</v>
       </c>
       <c r="L378" s="2" t="inlineStr"/>
+      <c r="M378" s="2" t="inlineStr">
+        <is>
+          <t>reigate.boltguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="379">
       <c r="A379" s="2" t="inlineStr">
@@ -17968,6 +19490,11 @@
         <v>23</v>
       </c>
       <c r="L379" s="2" t="inlineStr"/>
+      <c r="M379" s="2" t="inlineStr">
+        <is>
+          <t>tadworth.lockguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="380">
       <c r="A380" s="2" t="inlineStr">
@@ -18014,6 +19541,11 @@
         <v>23</v>
       </c>
       <c r="L380" s="2" t="inlineStr"/>
+      <c r="M380" s="2" t="inlineStr">
+        <is>
+          <t>walton-on-thames.lockguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="381">
       <c r="A381" s="2" t="inlineStr">
@@ -18060,6 +19592,11 @@
         <v>23</v>
       </c>
       <c r="L381" s="2" t="inlineStr"/>
+      <c r="M381" s="2" t="inlineStr">
+        <is>
+          <t>west-molesey.lockguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="382">
       <c r="A382" s="2" t="inlineStr">
@@ -18106,6 +19643,11 @@
         <v>21</v>
       </c>
       <c r="L382" s="2" t="inlineStr"/>
+      <c r="M382" s="2" t="inlineStr">
+        <is>
+          <t>chippenham.vaultlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="383">
       <c r="A383" s="2" t="inlineStr">
@@ -18152,6 +19694,11 @@
         <v>21</v>
       </c>
       <c r="L383" s="2" t="inlineStr"/>
+      <c r="M383" s="2" t="inlineStr">
+        <is>
+          <t>christchurch.vaultlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="384">
       <c r="A384" s="2" t="inlineStr">
@@ -18198,6 +19745,11 @@
         <v>21</v>
       </c>
       <c r="L384" s="2" t="inlineStr"/>
+      <c r="M384" s="2" t="inlineStr">
+        <is>
+          <t>clevedon.vaultlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="385">
       <c r="A385" s="2" t="inlineStr">
@@ -18244,6 +19796,11 @@
         <v>21</v>
       </c>
       <c r="L385" s="2" t="inlineStr"/>
+      <c r="M385" s="2" t="inlineStr">
+        <is>
+          <t>fishponds.vaultlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="386">
       <c r="A386" s="2" t="inlineStr">
@@ -18290,6 +19847,11 @@
         <v>21</v>
       </c>
       <c r="L386" s="2" t="inlineStr"/>
+      <c r="M386" s="2" t="inlineStr">
+        <is>
+          <t>frome.vaultlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="387">
       <c r="A387" s="2" t="inlineStr">
@@ -18336,6 +19898,11 @@
         <v>21</v>
       </c>
       <c r="L387" s="2" t="inlineStr"/>
+      <c r="M387" s="2" t="inlineStr">
+        <is>
+          <t>kingswood.vaultlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="388">
       <c r="A388" s="2" t="inlineStr">
@@ -18382,6 +19949,11 @@
         <v>21</v>
       </c>
       <c r="L388" s="2" t="inlineStr"/>
+      <c r="M388" s="2" t="inlineStr">
+        <is>
+          <t>portishead.vaultlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="389">
       <c r="A389" s="2" t="inlineStr">
@@ -18428,6 +20000,11 @@
         <v>21</v>
       </c>
       <c r="L389" s="2" t="inlineStr"/>
+      <c r="M389" s="2" t="inlineStr">
+        <is>
+          <t>yate.vaultlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="390">
       <c r="A390" s="2" t="inlineStr">
@@ -18474,6 +20051,11 @@
         <v>21</v>
       </c>
       <c r="L390" s="2" t="inlineStr"/>
+      <c r="M390" s="2" t="inlineStr">
+        <is>
+          <t>yeovil.vaultlok-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="391">
       <c r="A391" s="2" t="inlineStr">
@@ -18520,6 +20102,11 @@
         <v>26</v>
       </c>
       <c r="L391" s="2" t="inlineStr"/>
+      <c r="M391" s="2" t="inlineStr">
+        <is>
+          <t>crowborough.latchguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="392">
       <c r="A392" s="2" t="inlineStr">
@@ -18566,6 +20153,11 @@
         <v>22</v>
       </c>
       <c r="L392" s="2" t="inlineStr"/>
+      <c r="M392" s="2" t="inlineStr">
+        <is>
+          <t>deal.keyguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="393">
       <c r="A393" s="2" t="inlineStr">
@@ -18612,6 +20204,11 @@
         <v>22</v>
       </c>
       <c r="L393" s="2" t="inlineStr"/>
+      <c r="M393" s="2" t="inlineStr">
+        <is>
+          <t>folkestone.keyguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="394">
       <c r="A394" s="2" t="inlineStr">
@@ -18658,6 +20255,11 @@
         <v>26</v>
       </c>
       <c r="L394" s="2" t="inlineStr"/>
+      <c r="M394" s="2" t="inlineStr">
+        <is>
+          <t>hailsham.latchguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="395">
       <c r="A395" s="2" t="inlineStr">
@@ -18704,6 +20306,11 @@
         <v>26</v>
       </c>
       <c r="L395" s="2" t="inlineStr"/>
+      <c r="M395" s="2" t="inlineStr">
+        <is>
+          <t>haywards-heath.latchguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="396">
       <c r="A396" s="2" t="inlineStr">
@@ -18750,6 +20357,11 @@
         <v>24</v>
       </c>
       <c r="L396" s="2" t="inlineStr"/>
+      <c r="M396" s="2" t="inlineStr">
+        <is>
+          <t>horley.boltguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="397">
       <c r="A397" s="2" t="inlineStr">
@@ -18796,6 +20408,11 @@
         <v>24</v>
       </c>
       <c r="L397" s="2" t="inlineStr"/>
+      <c r="M397" s="2" t="inlineStr">
+        <is>
+          <t>royal-tunbridge-wells.boltguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="398">
       <c r="A398" s="2" t="inlineStr">
@@ -18842,6 +20459,11 @@
         <v>26</v>
       </c>
       <c r="L398" s="2" t="inlineStr"/>
+      <c r="M398" s="2" t="inlineStr">
+        <is>
+          <t>seaford.latchguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="399">
       <c r="A399" s="2" t="inlineStr">
@@ -18888,6 +20510,11 @@
         <v>24</v>
       </c>
       <c r="L399" s="2" t="inlineStr"/>
+      <c r="M399" s="2" t="inlineStr">
+        <is>
+          <t>tonbridge.boltguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="400">
       <c r="A400" s="2" t="inlineStr">
@@ -18934,6 +20561,11 @@
       </c>
       <c r="K400" s="2" t="inlineStr"/>
       <c r="L400" s="2" t="inlineStr"/>
+      <c r="M400" s="2" t="inlineStr">
+        <is>
+          <t>lockrootbognorregislocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="401">
       <c r="A401" s="2" t="inlineStr">
@@ -18980,6 +20612,11 @@
       </c>
       <c r="K401" s="2" t="inlineStr"/>
       <c r="L401" s="2" t="inlineStr"/>
+      <c r="M401" s="2" t="inlineStr">
+        <is>
+          <t>boltpointbrightonlocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="402">
       <c r="A402" s="2" t="inlineStr">
@@ -19026,6 +20663,11 @@
         <v>26</v>
       </c>
       <c r="L402" s="2" t="inlineStr"/>
+      <c r="M402" s="2" t="inlineStr">
+        <is>
+          <t>burgess-hill.latchguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="403">
       <c r="A403" s="2" t="inlineStr">
@@ -19072,6 +20714,11 @@
         <v>25</v>
       </c>
       <c r="L403" s="2" t="inlineStr"/>
+      <c r="M403" s="2" t="inlineStr">
+        <is>
+          <t>chichester.sureguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="404">
       <c r="A404" s="2" t="inlineStr">
@@ -19118,6 +20765,11 @@
         <v>25</v>
       </c>
       <c r="L404" s="2" t="inlineStr"/>
+      <c r="M404" s="2" t="inlineStr">
+        <is>
+          <t>hedge-end.sureguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="405">
       <c r="A405" s="2" t="inlineStr">
@@ -19164,6 +20816,11 @@
       </c>
       <c r="K405" s="2" t="inlineStr"/>
       <c r="L405" s="2" t="inlineStr"/>
+      <c r="M405" s="2" t="inlineStr">
+        <is>
+          <t>lockgridhovelocksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="406">
       <c r="A406" s="2" t="inlineStr">
@@ -19210,6 +20867,11 @@
         <v>26</v>
       </c>
       <c r="L406" s="2" t="inlineStr"/>
+      <c r="M406" s="2" t="inlineStr">
+        <is>
+          <t>portslade.latchguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="407">
       <c r="A407" s="2" t="inlineStr">
@@ -19256,6 +20918,11 @@
         <v>26</v>
       </c>
       <c r="L407" s="2" t="inlineStr"/>
+      <c r="M407" s="2" t="inlineStr">
+        <is>
+          <t>rustington.latchguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
     <row r="408">
       <c r="A408" s="2" t="inlineStr">
@@ -19302,9 +20969,14 @@
         <v>25</v>
       </c>
       <c r="L408" s="2" t="inlineStr"/>
+      <c r="M408" s="2" t="inlineStr">
+        <is>
+          <t>ryde.sureguard-locksmiths.co.uk</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L408"/>
+  <autoFilter ref="A1:M408"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19315,7 +20987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -19426,6 +21098,18 @@
       </c>
       <c r="B12" s="2" t="inlineStr"/>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr"/>
+    </row>
+    <row r="14" ht="60" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Domain suggestions: unique brand per site following fleet conventions; all 151 suggested domains returned NXDOMAIN on DNS check 2026-07-21 (verify at registrar). doorfix-locksmiths.co.uk (owned) assigned to Bundle 01.</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix apostrophe slug: bishop-s-stortford -> bishops-stortford
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018qYwdxW5238hQ6ii9dUE6c
</commit_message>
<xml_diff>
--- a/data/locksmith-fleet/coverage-plan-final.xlsx
+++ b/data/locksmith-fleet/coverage-plan-final.xlsx
@@ -16745,7 +16745,7 @@
     <row r="326">
       <c r="A326" s="2" t="inlineStr">
         <is>
-          <t>bishop-s-stortford</t>
+          <t>bishops-stortford</t>
         </is>
       </c>
       <c r="B326" s="2" t="inlineStr">
@@ -16789,7 +16789,7 @@
       <c r="L326" s="2" t="inlineStr"/>
       <c r="M326" s="2" t="inlineStr">
         <is>
-          <t>bishop-s-stortford.gatelok-locksmiths.co.uk</t>
+          <t>bishops-stortford.gatelok-locksmiths.co.uk</t>
         </is>
       </c>
     </row>
@@ -21098,17 +21098,13 @@
       </c>
       <c r="B12" s="2" t="inlineStr"/>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr"/>
-      <c r="B13" t="inlineStr"/>
-    </row>
+    <row r="13"/>
     <row r="14" ht="60" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
           <t>Domain suggestions: unique brand per site following fleet conventions; all 151 suggested domains returned NXDOMAIN on DNS check 2026-07-21 (verify at registrar). doorfix-locksmiths.co.uk (owned) assigned to Bundle 01.</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Vary individual-site domain structure across four formats
Same brand tokens, but domains now rotate evenly (32/32/31/31) through
brand+location+locksmiths, brand+location+locksmith,
brand+locksmith+location and brand+locksmiths+location so the fleet
does not share a single naming footprint. All re-checked via DNS.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018qYwdxW5238hQ6ii9dUE6c
</commit_message>
<xml_diff>
--- a/data/locksmith-fleet/coverage-plan-final.xlsx
+++ b/data/locksmith-fleet/coverage-plan-final.xlsx
@@ -811,7 +811,7 @@
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>boltrouteloughboroughlocksmiths.co.uk</t>
+          <t>boltroutelocksmithloughborough.co.uk</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>boltwavepeterboroughlocksmiths.co.uk</t>
+          <t>boltwavelocksmithpeterborough.co.uk</t>
         </is>
       </c>
     </row>
@@ -1663,7 +1663,7 @@
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>latchmaxgatesheadlocksmiths.co.uk</t>
+          <t>latchmaxlocksmithsgateshead.co.uk</t>
         </is>
       </c>
     </row>
@@ -2412,7 +2412,7 @@
       </c>
       <c r="M41" s="2" t="inlineStr">
         <is>
-          <t>lockcrewrochdalelocksmiths.co.uk</t>
+          <t>lockcrewrochdalelocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -2471,7 +2471,7 @@
       </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>boltsmartruncornlocksmiths.co.uk</t>
+          <t>boltsmartlocksmithruncorn.co.uk</t>
         </is>
       </c>
     </row>
@@ -2530,7 +2530,7 @@
       </c>
       <c r="M43" s="2" t="inlineStr">
         <is>
-          <t>lockjetwallaseylocksmiths.co.uk</t>
+          <t>lockjetwallaseylocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -2589,7 +2589,7 @@
       </c>
       <c r="M44" s="2" t="inlineStr">
         <is>
-          <t>boltpeakwarringtonlocksmiths.co.uk</t>
+          <t>boltpeaklocksmithwarrington.co.uk</t>
         </is>
       </c>
     </row>
@@ -2824,7 +2824,7 @@
       </c>
       <c r="M49" s="2" t="inlineStr">
         <is>
-          <t>bolthavenaylesburylocksmiths.co.uk</t>
+          <t>bolthavenlocksmithaylesbury.co.uk</t>
         </is>
       </c>
     </row>
@@ -3103,7 +3103,7 @@
       </c>
       <c r="M55" s="2" t="inlineStr">
         <is>
-          <t>latchsmartfarnboroughlocksmiths.co.uk</t>
+          <t>latchsmartlocksmithsfarnborough.co.uk</t>
         </is>
       </c>
     </row>
@@ -3250,7 +3250,7 @@
       </c>
       <c r="M58" s="2" t="inlineStr">
         <is>
-          <t>boltgridhastingslocksmiths.co.uk</t>
+          <t>boltgridlocksmithhastings.co.uk</t>
         </is>
       </c>
     </row>
@@ -3485,7 +3485,7 @@
       </c>
       <c r="M63" s="2" t="inlineStr">
         <is>
-          <t>latchpeakoxfordlocksmiths.co.uk</t>
+          <t>latchpeaklocksmithsoxford.co.uk</t>
         </is>
       </c>
     </row>
@@ -3588,7 +3588,7 @@
       </c>
       <c r="M65" s="2" t="inlineStr">
         <is>
-          <t>lockpointsloughlocksmiths.co.uk</t>
+          <t>lockpointsloughlocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -3735,7 +3735,7 @@
       </c>
       <c r="M68" s="2" t="inlineStr">
         <is>
-          <t>latchpulsewokinglocksmiths.co.uk</t>
+          <t>latchpulselocksmithswoking.co.uk</t>
         </is>
       </c>
     </row>
@@ -3853,7 +3853,7 @@
       </c>
       <c r="M70" s="2" t="inlineStr">
         <is>
-          <t>lockwavebournemouthlocksmiths.co.uk</t>
+          <t>lockwavebournemouthlocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
       </c>
       <c r="M73" s="2" t="inlineStr">
         <is>
-          <t>lockmaxcheltenhamlocksmiths.co.uk</t>
+          <t>lockmaxcheltenhamlocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -4323,7 +4323,7 @@
       </c>
       <c r="M80" s="2" t="inlineStr">
         <is>
-          <t>lockpulseburtonontrentlocksmiths.co.uk</t>
+          <t>lockpulseburtonontrentlocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -4602,7 +4602,7 @@
       </c>
       <c r="M86" s="2" t="inlineStr">
         <is>
-          <t>latchstarstokeontrentlocksmiths.co.uk</t>
+          <t>latchstarlocksmithsstokeontrent.co.uk</t>
         </is>
       </c>
     </row>
@@ -4661,7 +4661,7 @@
       </c>
       <c r="M87" s="2" t="inlineStr">
         <is>
-          <t>boltpulsetamworthlocksmiths.co.uk</t>
+          <t>boltpulselocksmithtamworth.co.uk</t>
         </is>
       </c>
     </row>
@@ -4940,7 +4940,7 @@
       </c>
       <c r="M93" s="2" t="inlineStr">
         <is>
-          <t>latchhavendoncasterlocksmiths.co.uk</t>
+          <t>latchhavenlocksmithsdoncaster.co.uk</t>
         </is>
       </c>
     </row>
@@ -5365,7 +5365,7 @@
       <c r="L102" s="2" t="inlineStr"/>
       <c r="M102" s="2" t="inlineStr">
         <is>
-          <t>lockstarderbylocksmiths.co.uk</t>
+          <t>lockstarderbylocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -5467,7 +5467,7 @@
       <c r="L104" s="2" t="inlineStr"/>
       <c r="M104" s="2" t="inlineStr">
         <is>
-          <t>boltmaxbasildonlocksmiths.co.uk</t>
+          <t>boltmaxlocksmithbasildon.co.uk</t>
         </is>
       </c>
     </row>
@@ -5518,7 +5518,7 @@
       <c r="L105" s="2" t="inlineStr"/>
       <c r="M105" s="2" t="inlineStr">
         <is>
-          <t>latchedgebedfordlocksmiths.co.uk</t>
+          <t>latchedgelocksmithsbedford.co.uk</t>
         </is>
       </c>
     </row>
@@ -5569,7 +5569,7 @@
       <c r="L106" s="2" t="inlineStr"/>
       <c r="M106" s="2" t="inlineStr">
         <is>
-          <t>boltspotbraintreelocksmiths.co.uk</t>
+          <t>boltspotlocksmithbraintree.co.uk</t>
         </is>
       </c>
     </row>
@@ -5671,7 +5671,7 @@
       <c r="L108" s="2" t="inlineStr"/>
       <c r="M108" s="2" t="inlineStr">
         <is>
-          <t>latchcrewchelmsfordlocksmiths.co.uk</t>
+          <t>latchcrewlocksmithschelmsford.co.uk</t>
         </is>
       </c>
     </row>
@@ -5722,7 +5722,7 @@
       <c r="L109" s="2" t="inlineStr"/>
       <c r="M109" s="2" t="inlineStr">
         <is>
-          <t>latchlinkcolchesterlocksmiths.co.uk</t>
+          <t>latchlinklocksmithscolchester.co.uk</t>
         </is>
       </c>
     </row>
@@ -5773,7 +5773,7 @@
       <c r="L110" s="2" t="inlineStr"/>
       <c r="M110" s="2" t="inlineStr">
         <is>
-          <t>lockgateharlowlocksmiths.co.uk</t>
+          <t>lockgateharlowlocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -5824,7 +5824,7 @@
       <c r="L111" s="2" t="inlineStr"/>
       <c r="M111" s="2" t="inlineStr">
         <is>
-          <t>locklineipswichlocksmiths.co.uk</t>
+          <t>locklineipswichlocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -5875,7 +5875,7 @@
       <c r="L112" s="2" t="inlineStr"/>
       <c r="M112" s="2" t="inlineStr">
         <is>
-          <t>boltzonelutonlocksmiths.co.uk</t>
+          <t>boltzonelocksmithluton.co.uk</t>
         </is>
       </c>
     </row>
@@ -5926,7 +5926,7 @@
       <c r="L113" s="2" t="inlineStr"/>
       <c r="M113" s="2" t="inlineStr">
         <is>
-          <t>lockpeaksouthendlocksmiths.co.uk</t>
+          <t>lockpeaksouthendlocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -5977,7 +5977,7 @@
       <c r="L114" s="2" t="inlineStr"/>
       <c r="M114" s="2" t="inlineStr">
         <is>
-          <t>boltcorestevenagelocksmiths.co.uk</t>
+          <t>boltcorelocksmithstevenage.co.uk</t>
         </is>
       </c>
     </row>
@@ -6028,7 +6028,7 @@
       <c r="L115" s="2" t="inlineStr"/>
       <c r="M115" s="2" t="inlineStr">
         <is>
-          <t>latchgatedarlingtonlocksmiths.co.uk</t>
+          <t>latchgatelocksmithsdarlington.co.uk</t>
         </is>
       </c>
     </row>
@@ -6079,7 +6079,7 @@
       <c r="L116" s="2" t="inlineStr"/>
       <c r="M116" s="2" t="inlineStr">
         <is>
-          <t>lockhavenhartlepoollocksmiths.co.uk</t>
+          <t>lockhavenhartlepoollocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -6130,7 +6130,7 @@
       <c r="L117" s="2" t="inlineStr"/>
       <c r="M117" s="2" t="inlineStr">
         <is>
-          <t>boltlinemiddlesbroughlocksmiths.co.uk</t>
+          <t>boltlinelocksmithmiddlesbrough.co.uk</t>
         </is>
       </c>
     </row>
@@ -6232,7 +6232,7 @@
       <c r="L119" s="2" t="inlineStr"/>
       <c r="M119" s="2" t="inlineStr">
         <is>
-          <t>boltjetstocktonlocksmiths.co.uk</t>
+          <t>boltjetlocksmithstockton.co.uk</t>
         </is>
       </c>
     </row>
@@ -6283,7 +6283,7 @@
       <c r="L120" s="2" t="inlineStr"/>
       <c r="M120" s="2" t="inlineStr">
         <is>
-          <t>latchwaveboltonlocksmiths.co.uk</t>
+          <t>latchwavelocksmithsbolton.co.uk</t>
         </is>
       </c>
     </row>
@@ -6385,7 +6385,7 @@
       <c r="L122" s="2" t="inlineStr"/>
       <c r="M122" s="2" t="inlineStr">
         <is>
-          <t>boltcrewoldhamlocksmiths.co.uk</t>
+          <t>boltcrewlocksmitholdham.co.uk</t>
         </is>
       </c>
     </row>
@@ -6436,7 +6436,7 @@
       <c r="L123" s="2" t="inlineStr"/>
       <c r="M123" s="2" t="inlineStr">
         <is>
-          <t>lockcoreprestonlocksmiths.co.uk</t>
+          <t>lockcoreprestonlocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -6487,7 +6487,7 @@
       <c r="L124" s="2" t="inlineStr"/>
       <c r="M124" s="2" t="inlineStr">
         <is>
-          <t>latchcraftsalfordlocksmiths.co.uk</t>
+          <t>latchcraftlocksmithssalford.co.uk</t>
         </is>
       </c>
     </row>
@@ -6538,7 +6538,7 @@
       <c r="L125" s="2" t="inlineStr"/>
       <c r="M125" s="2" t="inlineStr">
         <is>
-          <t>latchmatestockportlocksmiths.co.uk</t>
+          <t>latchmatelocksmithsstockport.co.uk</t>
         </is>
       </c>
     </row>
@@ -6589,7 +6589,7 @@
       <c r="L126" s="2" t="inlineStr"/>
       <c r="M126" s="2" t="inlineStr">
         <is>
-          <t>latchkingwiganlocksmiths.co.uk</t>
+          <t>latchkinglocksmithswigan.co.uk</t>
         </is>
       </c>
     </row>
@@ -6640,7 +6640,7 @@
       <c r="L127" s="2" t="inlineStr"/>
       <c r="M127" s="2" t="inlineStr">
         <is>
-          <t>lockkingashfordlocksmiths.co.uk</t>
+          <t>lockkingashfordlocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -6691,7 +6691,7 @@
       <c r="L128" s="2" t="inlineStr"/>
       <c r="M128" s="2" t="inlineStr">
         <is>
-          <t>boltsparkcanterburylocksmiths.co.uk</t>
+          <t>boltsparklocksmithcanterbury.co.uk</t>
         </is>
       </c>
     </row>
@@ -6742,7 +6742,7 @@
       <c r="L129" s="2" t="inlineStr"/>
       <c r="M129" s="2" t="inlineStr">
         <is>
-          <t>lockmatecrawleylocksmiths.co.uk</t>
+          <t>lockmatecrawleylocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -6793,7 +6793,7 @@
       <c r="L130" s="2" t="inlineStr"/>
       <c r="M130" s="2" t="inlineStr">
         <is>
-          <t>boltsprintdoverlocksmiths.co.uk</t>
+          <t>boltsprintlocksmithdover.co.uk</t>
         </is>
       </c>
     </row>
@@ -6895,7 +6895,7 @@
       <c r="L132" s="2" t="inlineStr"/>
       <c r="M132" s="2" t="inlineStr">
         <is>
-          <t>latchspotfarehamlocksmiths.co.uk</t>
+          <t>latchspotlocksmithsfareham.co.uk</t>
         </is>
       </c>
     </row>
@@ -6946,7 +6946,7 @@
       <c r="L133" s="2" t="inlineStr"/>
       <c r="M133" s="2" t="inlineStr">
         <is>
-          <t>boltcraftgillinghamlocksmiths.co.uk</t>
+          <t>boltcraftlocksmithgillingham.co.uk</t>
         </is>
       </c>
     </row>
@@ -6997,7 +6997,7 @@
       <c r="L134" s="2" t="inlineStr"/>
       <c r="M134" s="2" t="inlineStr">
         <is>
-          <t>locknestguildfordlocksmiths.co.uk</t>
+          <t>locknestguildfordlocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -7099,7 +7099,7 @@
       <c r="L136" s="2" t="inlineStr"/>
       <c r="M136" s="2" t="inlineStr">
         <is>
-          <t>lockcraftmaidstonelocksmiths.co.uk</t>
+          <t>lockcraftmaidstonelocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -7201,7 +7201,7 @@
       <c r="L138" s="2" t="inlineStr"/>
       <c r="M138" s="2" t="inlineStr">
         <is>
-          <t>latchzonereadinglocksmiths.co.uk</t>
+          <t>latchzonelocksmithsreading.co.uk</t>
         </is>
       </c>
     </row>
@@ -7252,7 +7252,7 @@
       <c r="L139" s="2" t="inlineStr"/>
       <c r="M139" s="2" t="inlineStr">
         <is>
-          <t>lockspotwinchesterlocksmiths.co.uk</t>
+          <t>lockspotwinchesterlocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -7303,7 +7303,7 @@
       <c r="L140" s="2" t="inlineStr"/>
       <c r="M140" s="2" t="inlineStr">
         <is>
-          <t>latchsparkwokinghamlocksmiths.co.uk</t>
+          <t>latchsparklocksmithswokingham.co.uk</t>
         </is>
       </c>
     </row>
@@ -7405,7 +7405,7 @@
       <c r="L142" s="2" t="inlineStr"/>
       <c r="M142" s="2" t="inlineStr">
         <is>
-          <t>boltmategloucesterlocksmiths.co.uk</t>
+          <t>boltmatelocksmithgloucester.co.uk</t>
         </is>
       </c>
     </row>
@@ -7456,7 +7456,7 @@
       <c r="L143" s="2" t="inlineStr"/>
       <c r="M143" s="2" t="inlineStr">
         <is>
-          <t>locklinkpoolelocksmiths.co.uk</t>
+          <t>locklinkpoolelocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -7507,7 +7507,7 @@
       <c r="L144" s="2" t="inlineStr"/>
       <c r="M144" s="2" t="inlineStr">
         <is>
-          <t>locksquadstroudlocksmiths.co.uk</t>
+          <t>locksquadstroudlocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -7558,7 +7558,7 @@
       <c r="L145" s="2" t="inlineStr"/>
       <c r="M145" s="2" t="inlineStr">
         <is>
-          <t>latchjetwestonsupermarelocksmiths.co.uk</t>
+          <t>latchjetlocksmithswestonsupermare.co.uk</t>
         </is>
       </c>
     </row>
@@ -7609,7 +7609,7 @@
       <c r="L146" s="2" t="inlineStr"/>
       <c r="M146" s="2" t="inlineStr">
         <is>
-          <t>latchroutedudleylocksmiths.co.uk</t>
+          <t>latchroutelocksmithsdudley.co.uk</t>
         </is>
       </c>
     </row>
@@ -7660,7 +7660,7 @@
       <c r="L147" s="2" t="inlineStr"/>
       <c r="M147" s="2" t="inlineStr">
         <is>
-          <t>latchsprintlichfieldlocksmiths.co.uk</t>
+          <t>latchsprintlocksmithslichfield.co.uk</t>
         </is>
       </c>
     </row>
@@ -7711,7 +7711,7 @@
       <c r="L148" s="2" t="inlineStr"/>
       <c r="M148" s="2" t="inlineStr">
         <is>
-          <t>latchnestnewcastleunderlymelocksmiths.co.uk</t>
+          <t>latchnestlocksmithsnewcastleunderlyme.co.uk</t>
         </is>
       </c>
     </row>
@@ -7762,7 +7762,7 @@
       <c r="L149" s="2" t="inlineStr"/>
       <c r="M149" s="2" t="inlineStr">
         <is>
-          <t>boltkingredditchlocksmiths.co.uk</t>
+          <t>boltkinglocksmithredditch.co.uk</t>
         </is>
       </c>
     </row>
@@ -7813,7 +7813,7 @@
       <c r="L150" s="2" t="inlineStr"/>
       <c r="M150" s="2" t="inlineStr">
         <is>
-          <t>boltgatesuttoncoldfieldlocksmiths.co.uk</t>
+          <t>boltgatelocksmithsuttoncoldfield.co.uk</t>
         </is>
       </c>
     </row>
@@ -8017,7 +8017,7 @@
       <c r="L154" s="2" t="inlineStr"/>
       <c r="M154" s="2" t="inlineStr">
         <is>
-          <t>latchrisewalsalllocksmiths.co.uk</t>
+          <t>latchriselocksmithswalsall.co.uk</t>
         </is>
       </c>
     </row>
@@ -8068,7 +8068,7 @@
       <c r="L155" s="2" t="inlineStr"/>
       <c r="M155" s="2" t="inlineStr">
         <is>
-          <t>locksprintwarwicklocksmiths.co.uk</t>
+          <t>locksprintwarwicklocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -8119,7 +8119,7 @@
       <c r="L156" s="2" t="inlineStr"/>
       <c r="M156" s="2" t="inlineStr">
         <is>
-          <t>lockzonewolverhamptonlocksmiths.co.uk</t>
+          <t>lockzonewolverhamptonlocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -8170,7 +8170,7 @@
       <c r="L157" s="2" t="inlineStr"/>
       <c r="M157" s="2" t="inlineStr">
         <is>
-          <t>boltdashworcesterlocksmiths.co.uk</t>
+          <t>boltdashlocksmithworcester.co.uk</t>
         </is>
       </c>
     </row>
@@ -8221,7 +8221,7 @@
       <c r="L158" s="2" t="inlineStr"/>
       <c r="M158" s="2" t="inlineStr">
         <is>
-          <t>boltrisebarnsleylocksmiths.co.uk</t>
+          <t>boltriselocksmithbarnsley.co.uk</t>
         </is>
       </c>
     </row>
@@ -8272,7 +8272,7 @@
       <c r="L159" s="2" t="inlineStr"/>
       <c r="M159" s="2" t="inlineStr">
         <is>
-          <t>lockquestharrogatelocksmiths.co.uk</t>
+          <t>lockquestharrogatelocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -8323,7 +8323,7 @@
       <c r="L160" s="2" t="inlineStr"/>
       <c r="M160" s="2" t="inlineStr">
         <is>
-          <t>boltstarhulllocksmiths.co.uk</t>
+          <t>boltstarlocksmithhull.co.uk</t>
         </is>
       </c>
     </row>
@@ -8425,7 +8425,7 @@
       <c r="L162" s="2" t="inlineStr"/>
       <c r="M162" s="2" t="inlineStr">
         <is>
-          <t>lockriserotherhamlocksmiths.co.uk</t>
+          <t>lockriserotherhamlocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -8476,7 +8476,7 @@
       <c r="L163" s="2" t="inlineStr"/>
       <c r="M163" s="2" t="inlineStr">
         <is>
-          <t>lockedgewakefieldlocksmiths.co.uk</t>
+          <t>lockedgewakefieldlocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -8527,7 +8527,7 @@
       <c r="L164" s="2" t="inlineStr"/>
       <c r="M164" s="2" t="inlineStr">
         <is>
-          <t>latchlineyorklocksmiths.co.uk</t>
+          <t>latchlinelocksmithsyork.co.uk</t>
         </is>
       </c>
     </row>
@@ -8884,7 +8884,7 @@
       <c r="L171" s="2" t="inlineStr"/>
       <c r="M171" s="2" t="inlineStr">
         <is>
-          <t>latchquestsouthshieldslocksmiths.co.uk</t>
+          <t>latchquestlocksmithssouthshields.co.uk</t>
         </is>
       </c>
     </row>
@@ -9700,7 +9700,7 @@
       <c r="L187" s="2" t="inlineStr"/>
       <c r="M187" s="2" t="inlineStr">
         <is>
-          <t>latchnodeburnleylocksmiths.co.uk</t>
+          <t>latchnodelocksmithsburnley.co.uk</t>
         </is>
       </c>
     </row>
@@ -9751,7 +9751,7 @@
       <c r="L188" s="2" t="inlineStr"/>
       <c r="M188" s="2" t="inlineStr">
         <is>
-          <t>locknodeburylocksmiths.co.uk</t>
+          <t>locknodeburylocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -10567,7 +10567,7 @@
       <c r="L204" s="2" t="inlineStr"/>
       <c r="M204" s="2" t="inlineStr">
         <is>
-          <t>latchcoresouthportlocksmiths.co.uk</t>
+          <t>latchcorelocksmithssouthport.co.uk</t>
         </is>
       </c>
     </row>
@@ -12301,7 +12301,7 @@
       <c r="L238" s="2" t="inlineStr"/>
       <c r="M238" s="2" t="inlineStr">
         <is>
-          <t>lockrouteellesmereportlocksmiths.co.uk</t>
+          <t>lockrouteellesmereportlocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -12556,7 +12556,7 @@
       <c r="L243" s="2" t="inlineStr"/>
       <c r="M243" s="2" t="inlineStr">
         <is>
-          <t>lockdashsthelenslocksmiths.co.uk</t>
+          <t>lockdashsthelenslocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -12862,7 +12862,7 @@
       <c r="L249" s="2" t="inlineStr"/>
       <c r="M249" s="2" t="inlineStr">
         <is>
-          <t>boltquestcrewelocksmiths.co.uk</t>
+          <t>boltquestlocksmithcrewe.co.uk</t>
         </is>
       </c>
     </row>
@@ -13015,7 +13015,7 @@
       <c r="L252" s="2" t="inlineStr"/>
       <c r="M252" s="2" t="inlineStr">
         <is>
-          <t>locksmartsalelocksmiths.co.uk</t>
+          <t>locksmartsalelocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -13117,7 +13117,7 @@
       <c r="L254" s="2" t="inlineStr"/>
       <c r="M254" s="2" t="inlineStr">
         <is>
-          <t>boltedgewythenshawelocksmiths.co.uk</t>
+          <t>boltedgelocksmithwythenshawe.co.uk</t>
         </is>
       </c>
     </row>
@@ -13525,7 +13525,7 @@
       <c r="L262" s="2" t="inlineStr"/>
       <c r="M262" s="2" t="inlineStr">
         <is>
-          <t>lockservemansfieldlocksmiths.co.uk</t>
+          <t>lockservemansfieldlocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -13780,7 +13780,7 @@
       <c r="L267" s="2" t="inlineStr"/>
       <c r="M267" s="2" t="inlineStr">
         <is>
-          <t>boltrootcorbylocksmiths.co.uk</t>
+          <t>boltrootlocksmithcorby.co.uk</t>
         </is>
       </c>
     </row>
@@ -14443,7 +14443,7 @@
       <c r="L280" s="2" t="inlineStr"/>
       <c r="M280" s="2" t="inlineStr">
         <is>
-          <t>latchgridnuneatonlocksmiths.co.uk</t>
+          <t>latchgridlocksmithsnuneaton.co.uk</t>
         </is>
       </c>
     </row>
@@ -14647,7 +14647,7 @@
       <c r="L284" s="2" t="inlineStr"/>
       <c r="M284" s="2" t="inlineStr">
         <is>
-          <t>latchdashwestbromwichlocksmiths.co.uk</t>
+          <t>latchdashlocksmithswestbromwich.co.uk</t>
         </is>
       </c>
     </row>
@@ -15055,7 +15055,7 @@
       <c r="L292" s="2" t="inlineStr"/>
       <c r="M292" s="2" t="inlineStr">
         <is>
-          <t>latchpointtelfordlocksmiths.co.uk</t>
+          <t>latchpointlocksmithstelford.co.uk</t>
         </is>
       </c>
     </row>
@@ -15208,7 +15208,7 @@
       <c r="L295" s="2" t="inlineStr"/>
       <c r="M295" s="2" t="inlineStr">
         <is>
-          <t>latchserveketteringlocksmiths.co.uk</t>
+          <t>latchservelocksmithskettering.co.uk</t>
         </is>
       </c>
     </row>
@@ -15973,7 +15973,7 @@
       <c r="L310" s="2" t="inlineStr"/>
       <c r="M310" s="2" t="inlineStr">
         <is>
-          <t>locksparkhalesowenlocksmiths.co.uk</t>
+          <t>locksparkhalesowenlocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -16585,7 +16585,7 @@
       <c r="L322" s="2" t="inlineStr"/>
       <c r="M322" s="2" t="inlineStr">
         <is>
-          <t>boltlinkwatfordlocksmiths.co.uk</t>
+          <t>boltlinklocksmithwatford.co.uk</t>
         </is>
       </c>
     </row>
@@ -17605,7 +17605,7 @@
       <c r="L342" s="2" t="inlineStr"/>
       <c r="M342" s="2" t="inlineStr">
         <is>
-          <t>boltservemargatelocksmiths.co.uk</t>
+          <t>boltservelocksmithmargate.co.uk</t>
         </is>
       </c>
     </row>
@@ -18370,7 +18370,7 @@
       <c r="L357" s="2" t="inlineStr"/>
       <c r="M357" s="2" t="inlineStr">
         <is>
-          <t>boltnestchathamlocksmiths.co.uk</t>
+          <t>boltnestlocksmithchatham.co.uk</t>
         </is>
       </c>
     </row>
@@ -18778,7 +18778,7 @@
       <c r="L365" s="2" t="inlineStr"/>
       <c r="M365" s="2" t="inlineStr">
         <is>
-          <t>boltnodebracknelllocksmiths.co.uk</t>
+          <t>boltnodelocksmithbracknell.co.uk</t>
         </is>
       </c>
     </row>
@@ -18931,7 +18931,7 @@
       <c r="L368" s="2" t="inlineStr"/>
       <c r="M368" s="2" t="inlineStr">
         <is>
-          <t>latchrootmaidenheadlocksmiths.co.uk</t>
+          <t>latchrootlocksmithsmaidenhead.co.uk</t>
         </is>
       </c>
     </row>
@@ -20563,7 +20563,7 @@
       <c r="L400" s="2" t="inlineStr"/>
       <c r="M400" s="2" t="inlineStr">
         <is>
-          <t>lockrootbognorregislocksmiths.co.uk</t>
+          <t>lockrootbognorregislocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -20614,7 +20614,7 @@
       <c r="L401" s="2" t="inlineStr"/>
       <c r="M401" s="2" t="inlineStr">
         <is>
-          <t>boltpointbrightonlocksmiths.co.uk</t>
+          <t>boltpointlocksmithbrighton.co.uk</t>
         </is>
       </c>
     </row>
@@ -20818,7 +20818,7 @@
       <c r="L405" s="2" t="inlineStr"/>
       <c r="M405" s="2" t="inlineStr">
         <is>
-          <t>lockgridhovelocksmiths.co.uk</t>
+          <t>lockgridhovelocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -21098,7 +21098,6 @@
       </c>
       <c r="B12" s="2" t="inlineStr"/>
     </row>
-    <row r="13"/>
     <row r="14" ht="60" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Mix hyphenation styles into individual-site domains
Four hyphenation styles (none, full, after-brand, before-last) now cycle
across the four word orders - 16 domain shapes spread evenly over the
126 individual sites. All changed domains re-checked via DNS.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018qYwdxW5238hQ6ii9dUE6c
</commit_message>
<xml_diff>
--- a/data/locksmith-fleet/coverage-plan-final.xlsx
+++ b/data/locksmith-fleet/coverage-plan-final.xlsx
@@ -811,7 +811,7 @@
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>boltroutelocksmithloughborough.co.uk</t>
+          <t>boltroute-locksmith-loughborough.co.uk</t>
         </is>
       </c>
     </row>
@@ -1134,7 +1134,7 @@
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>keycorehemelhempsteadlocksmiths.co.uk</t>
+          <t>keycore-hemelhempstead-locksmiths.co.uk</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>boltwavelocksmithpeterborough.co.uk</t>
+          <t>boltwave-locksmithpeterborough.co.uk</t>
         </is>
       </c>
     </row>
@@ -1340,7 +1340,7 @@
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>keyqueststalbanslocksmiths.co.uk</t>
+          <t>keyquest-stalbanslocksmiths.co.uk</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>keygridchesterlocksmiths.co.uk</t>
+          <t>keygridchester-locksmiths.co.uk</t>
         </is>
       </c>
     </row>
@@ -2412,7 +2412,7 @@
       </c>
       <c r="M41" s="2" t="inlineStr">
         <is>
-          <t>lockcrewrochdalelocksmith.co.uk</t>
+          <t>lockcrew-rochdale-locksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -2471,7 +2471,7 @@
       </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>boltsmartlocksmithruncorn.co.uk</t>
+          <t>boltsmartlocksmith-runcorn.co.uk</t>
         </is>
       </c>
     </row>
@@ -2530,7 +2530,7 @@
       </c>
       <c r="M43" s="2" t="inlineStr">
         <is>
-          <t>lockjetwallaseylocksmith.co.uk</t>
+          <t>lockjet-wallasey-locksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -2589,7 +2589,7 @@
       </c>
       <c r="M44" s="2" t="inlineStr">
         <is>
-          <t>boltpeaklocksmithwarrington.co.uk</t>
+          <t>boltpeaklocksmith-warrington.co.uk</t>
         </is>
       </c>
     </row>
@@ -3103,7 +3103,7 @@
       </c>
       <c r="M55" s="2" t="inlineStr">
         <is>
-          <t>latchsmartlocksmithsfarnborough.co.uk</t>
+          <t>latchsmartlocksmiths-farnborough.co.uk</t>
         </is>
       </c>
     </row>
@@ -3250,7 +3250,7 @@
       </c>
       <c r="M58" s="2" t="inlineStr">
         <is>
-          <t>boltgridlocksmithhastings.co.uk</t>
+          <t>boltgridlocksmith-hastings.co.uk</t>
         </is>
       </c>
     </row>
@@ -3485,7 +3485,7 @@
       </c>
       <c r="M63" s="2" t="inlineStr">
         <is>
-          <t>latchpeaklocksmithsoxford.co.uk</t>
+          <t>latchpeaklocksmiths-oxford.co.uk</t>
         </is>
       </c>
     </row>
@@ -3735,7 +3735,7 @@
       </c>
       <c r="M68" s="2" t="inlineStr">
         <is>
-          <t>latchpulselocksmithswoking.co.uk</t>
+          <t>latchpulse-locksmiths-woking.co.uk</t>
         </is>
       </c>
     </row>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="M69" s="2" t="inlineStr">
         <is>
-          <t>keycrewworthinglocksmiths.co.uk</t>
+          <t>keycrew-worthing-locksmiths.co.uk</t>
         </is>
       </c>
     </row>
@@ -3853,7 +3853,7 @@
       </c>
       <c r="M70" s="2" t="inlineStr">
         <is>
-          <t>lockwavebournemouthlocksmith.co.uk</t>
+          <t>lockwave-bournemouthlocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -4323,7 +4323,7 @@
       </c>
       <c r="M80" s="2" t="inlineStr">
         <is>
-          <t>lockpulseburtonontrentlocksmith.co.uk</t>
+          <t>lockpulse-burtonontrent-locksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -4661,7 +4661,7 @@
       </c>
       <c r="M87" s="2" t="inlineStr">
         <is>
-          <t>boltpulselocksmithtamworth.co.uk</t>
+          <t>boltpulse-locksmith-tamworth.co.uk</t>
         </is>
       </c>
     </row>
@@ -4999,7 +4999,7 @@
       </c>
       <c r="M94" s="2" t="inlineStr">
         <is>
-          <t>keyjetgrimsbylocksmiths.co.uk</t>
+          <t>keyjet-grimsby-locksmiths.co.uk</t>
         </is>
       </c>
     </row>
@@ -5314,7 +5314,7 @@
       <c r="L101" s="2" t="inlineStr"/>
       <c r="M101" s="2" t="inlineStr">
         <is>
-          <t>keypulsechesterfieldlocksmiths.co.uk</t>
+          <t>keypulse-chesterfield-locksmiths.co.uk</t>
         </is>
       </c>
     </row>
@@ -5416,7 +5416,7 @@
       <c r="L103" s="2" t="inlineStr"/>
       <c r="M103" s="2" t="inlineStr">
         <is>
-          <t>keyzonenorthamptonlocksmiths.co.uk</t>
+          <t>keyzone-northampton-locksmiths.co.uk</t>
         </is>
       </c>
     </row>
@@ -5569,7 +5569,7 @@
       <c r="L106" s="2" t="inlineStr"/>
       <c r="M106" s="2" t="inlineStr">
         <is>
-          <t>boltspotlocksmithbraintree.co.uk</t>
+          <t>boltspot-locksmith-braintree.co.uk</t>
         </is>
       </c>
     </row>
@@ -5620,7 +5620,7 @@
       <c r="L107" s="2" t="inlineStr"/>
       <c r="M107" s="2" t="inlineStr">
         <is>
-          <t>keylinecambridgelocksmiths.co.uk</t>
+          <t>keyline-cambridge-locksmiths.co.uk</t>
         </is>
       </c>
     </row>
@@ -5671,7 +5671,7 @@
       <c r="L108" s="2" t="inlineStr"/>
       <c r="M108" s="2" t="inlineStr">
         <is>
-          <t>latchcrewlocksmithschelmsford.co.uk</t>
+          <t>latchcrew-locksmiths-chelmsford.co.uk</t>
         </is>
       </c>
     </row>
@@ -5722,7 +5722,7 @@
       <c r="L109" s="2" t="inlineStr"/>
       <c r="M109" s="2" t="inlineStr">
         <is>
-          <t>latchlinklocksmithscolchester.co.uk</t>
+          <t>latchlink-locksmithscolchester.co.uk</t>
         </is>
       </c>
     </row>
@@ -5773,7 +5773,7 @@
       <c r="L110" s="2" t="inlineStr"/>
       <c r="M110" s="2" t="inlineStr">
         <is>
-          <t>lockgateharlowlocksmith.co.uk</t>
+          <t>lockgate-harlowlocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -5824,7 +5824,7 @@
       <c r="L111" s="2" t="inlineStr"/>
       <c r="M111" s="2" t="inlineStr">
         <is>
-          <t>locklineipswichlocksmith.co.uk</t>
+          <t>lockline-ipswich-locksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -5875,7 +5875,7 @@
       <c r="L112" s="2" t="inlineStr"/>
       <c r="M112" s="2" t="inlineStr">
         <is>
-          <t>boltzonelocksmithluton.co.uk</t>
+          <t>boltzone-locksmith-luton.co.uk</t>
         </is>
       </c>
     </row>
@@ -5926,7 +5926,7 @@
       <c r="L113" s="2" t="inlineStr"/>
       <c r="M113" s="2" t="inlineStr">
         <is>
-          <t>lockpeaksouthendlocksmith.co.uk</t>
+          <t>lockpeaksouthend-locksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -5977,7 +5977,7 @@
       <c r="L114" s="2" t="inlineStr"/>
       <c r="M114" s="2" t="inlineStr">
         <is>
-          <t>boltcorelocksmithstevenage.co.uk</t>
+          <t>boltcoretevenage-locksmith-stevenage.co.uk</t>
         </is>
       </c>
     </row>
@@ -6028,7 +6028,7 @@
       <c r="L115" s="2" t="inlineStr"/>
       <c r="M115" s="2" t="inlineStr">
         <is>
-          <t>latchgatelocksmithsdarlington.co.uk</t>
+          <t>latchgate-locksmithsdarlington.co.uk</t>
         </is>
       </c>
     </row>
@@ -6130,7 +6130,7 @@
       <c r="L117" s="2" t="inlineStr"/>
       <c r="M117" s="2" t="inlineStr">
         <is>
-          <t>boltlinelocksmithmiddlesbrough.co.uk</t>
+          <t>boltline-locksmith-middlesbrough.co.uk</t>
         </is>
       </c>
     </row>
@@ -6232,7 +6232,7 @@
       <c r="L119" s="2" t="inlineStr"/>
       <c r="M119" s="2" t="inlineStr">
         <is>
-          <t>boltjetlocksmithstockton.co.uk</t>
+          <t>boltjettockton-locksmith-stockton.co.uk</t>
         </is>
       </c>
     </row>
@@ -6283,7 +6283,7 @@
       <c r="L120" s="2" t="inlineStr"/>
       <c r="M120" s="2" t="inlineStr">
         <is>
-          <t>latchwavelocksmithsbolton.co.uk</t>
+          <t>latchwave-locksmithsbolton.co.uk</t>
         </is>
       </c>
     </row>
@@ -6334,7 +6334,7 @@
       <c r="L121" s="2" t="inlineStr"/>
       <c r="M121" s="2" t="inlineStr">
         <is>
-          <t>keysprintchorleylocksmiths.co.uk</t>
+          <t>keysprint-chorleylocksmiths.co.uk</t>
         </is>
       </c>
     </row>
@@ -6385,7 +6385,7 @@
       <c r="L122" s="2" t="inlineStr"/>
       <c r="M122" s="2" t="inlineStr">
         <is>
-          <t>boltcrewlocksmitholdham.co.uk</t>
+          <t>boltcrew-locksmith-oldham.co.uk</t>
         </is>
       </c>
     </row>
@@ -6436,7 +6436,7 @@
       <c r="L123" s="2" t="inlineStr"/>
       <c r="M123" s="2" t="inlineStr">
         <is>
-          <t>lockcoreprestonlocksmith.co.uk</t>
+          <t>lockcore-preston-locksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -6487,7 +6487,7 @@
       <c r="L124" s="2" t="inlineStr"/>
       <c r="M124" s="2" t="inlineStr">
         <is>
-          <t>latchcraftlocksmithssalford.co.uk</t>
+          <t>latchcraft-locksmithssalford.co.uk</t>
         </is>
       </c>
     </row>
@@ -6538,7 +6538,7 @@
       <c r="L125" s="2" t="inlineStr"/>
       <c r="M125" s="2" t="inlineStr">
         <is>
-          <t>latchmatelocksmithsstockport.co.uk</t>
+          <t>latchmatelocksmiths-stockport.co.uk</t>
         </is>
       </c>
     </row>
@@ -6589,7 +6589,7 @@
       <c r="L126" s="2" t="inlineStr"/>
       <c r="M126" s="2" t="inlineStr">
         <is>
-          <t>latchkinglocksmithswigan.co.uk</t>
+          <t>latchking-locksmithswigan.co.uk</t>
         </is>
       </c>
     </row>
@@ -6640,7 +6640,7 @@
       <c r="L127" s="2" t="inlineStr"/>
       <c r="M127" s="2" t="inlineStr">
         <is>
-          <t>lockkingashfordlocksmith.co.uk</t>
+          <t>lockking-ashfordlocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -6742,7 +6742,7 @@
       <c r="L129" s="2" t="inlineStr"/>
       <c r="M129" s="2" t="inlineStr">
         <is>
-          <t>lockmatecrawleylocksmith.co.uk</t>
+          <t>lockmatecrawley-locksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -6793,7 +6793,7 @@
       <c r="L130" s="2" t="inlineStr"/>
       <c r="M130" s="2" t="inlineStr">
         <is>
-          <t>boltsprintlocksmithdover.co.uk</t>
+          <t>boltsprint-locksmithdover.co.uk</t>
         </is>
       </c>
     </row>
@@ -6895,7 +6895,7 @@
       <c r="L132" s="2" t="inlineStr"/>
       <c r="M132" s="2" t="inlineStr">
         <is>
-          <t>latchspotlocksmithsfareham.co.uk</t>
+          <t>latchspot-locksmiths-fareham.co.uk</t>
         </is>
       </c>
     </row>
@@ -6946,7 +6946,7 @@
       <c r="L133" s="2" t="inlineStr"/>
       <c r="M133" s="2" t="inlineStr">
         <is>
-          <t>boltcraftlocksmithgillingham.co.uk</t>
+          <t>boltcraft-locksmithgillingham.co.uk</t>
         </is>
       </c>
     </row>
@@ -7048,7 +7048,7 @@
       <c r="L135" s="2" t="inlineStr"/>
       <c r="M135" s="2" t="inlineStr">
         <is>
-          <t>keyspothorshamlocksmiths.co.uk</t>
+          <t>keyspot-horsham-locksmiths.co.uk</t>
         </is>
       </c>
     </row>
@@ -7099,7 +7099,7 @@
       <c r="L136" s="2" t="inlineStr"/>
       <c r="M136" s="2" t="inlineStr">
         <is>
-          <t>lockcraftmaidstonelocksmith.co.uk</t>
+          <t>lockcraft-maidstonelocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -7150,7 +7150,7 @@
       <c r="L137" s="2" t="inlineStr"/>
       <c r="M137" s="2" t="inlineStr">
         <is>
-          <t>keywavemiltonkeyneslocksmiths.co.uk</t>
+          <t>keywave-miltonkeyneslocksmiths.co.uk</t>
         </is>
       </c>
     </row>
@@ -7201,7 +7201,7 @@
       <c r="L138" s="2" t="inlineStr"/>
       <c r="M138" s="2" t="inlineStr">
         <is>
-          <t>latchzonelocksmithsreading.co.uk</t>
+          <t>latchzone-locksmiths-reading.co.uk</t>
         </is>
       </c>
     </row>
@@ -7252,7 +7252,7 @@
       <c r="L139" s="2" t="inlineStr"/>
       <c r="M139" s="2" t="inlineStr">
         <is>
-          <t>lockspotwinchesterlocksmith.co.uk</t>
+          <t>lockspot-winchester-locksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -7354,7 +7354,7 @@
       <c r="L141" s="2" t="inlineStr"/>
       <c r="M141" s="2" t="inlineStr">
         <is>
-          <t>keygatebathlocksmiths.co.uk</t>
+          <t>keygate-bathlocksmiths.co.uk</t>
         </is>
       </c>
     </row>
@@ -7405,7 +7405,7 @@
       <c r="L142" s="2" t="inlineStr"/>
       <c r="M142" s="2" t="inlineStr">
         <is>
-          <t>boltmatelocksmithgloucester.co.uk</t>
+          <t>boltmatelocksmith-gloucester.co.uk</t>
         </is>
       </c>
     </row>
@@ -7456,7 +7456,7 @@
       <c r="L143" s="2" t="inlineStr"/>
       <c r="M143" s="2" t="inlineStr">
         <is>
-          <t>locklinkpoolelocksmith.co.uk</t>
+          <t>locklink-poolelocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -7507,7 +7507,7 @@
       <c r="L144" s="2" t="inlineStr"/>
       <c r="M144" s="2" t="inlineStr">
         <is>
-          <t>locksquadstroudlocksmith.co.uk</t>
+          <t>locksquadstroud-locksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -7558,7 +7558,7 @@
       <c r="L145" s="2" t="inlineStr"/>
       <c r="M145" s="2" t="inlineStr">
         <is>
-          <t>latchjetlocksmithswestonsupermare.co.uk</t>
+          <t>latchjet-locksmiths-westonsupermare.co.uk</t>
         </is>
       </c>
     </row>
@@ -7609,7 +7609,7 @@
       <c r="L146" s="2" t="inlineStr"/>
       <c r="M146" s="2" t="inlineStr">
         <is>
-          <t>latchroutelocksmithsdudley.co.uk</t>
+          <t>latchroute-locksmiths-dudley.co.uk</t>
         </is>
       </c>
     </row>
@@ -7660,7 +7660,7 @@
       <c r="L147" s="2" t="inlineStr"/>
       <c r="M147" s="2" t="inlineStr">
         <is>
-          <t>latchsprintlocksmithslichfield.co.uk</t>
+          <t>latchsprint-locksmithslichfield.co.uk</t>
         </is>
       </c>
     </row>
@@ -7762,7 +7762,7 @@
       <c r="L149" s="2" t="inlineStr"/>
       <c r="M149" s="2" t="inlineStr">
         <is>
-          <t>boltkinglocksmithredditch.co.uk</t>
+          <t>boltking-locksmithredditch.co.uk</t>
         </is>
       </c>
     </row>
@@ -7813,7 +7813,7 @@
       <c r="L150" s="2" t="inlineStr"/>
       <c r="M150" s="2" t="inlineStr">
         <is>
-          <t>boltgatelocksmithsuttoncoldfield.co.uk</t>
+          <t>boltgateuttoncoldfield-locksmithsuttoncoldfield.co.uk</t>
         </is>
       </c>
     </row>
@@ -7915,7 +7915,7 @@
       <c r="L152" s="2" t="inlineStr"/>
       <c r="M152" s="2" t="inlineStr">
         <is>
-          <t>keydashsolihulllocksmiths.co.uk</t>
+          <t>keydashsolihull-locksmiths.co.uk</t>
         </is>
       </c>
     </row>
@@ -7966,7 +7966,7 @@
       <c r="L153" s="2" t="inlineStr"/>
       <c r="M153" s="2" t="inlineStr">
         <is>
-          <t>keyrisestaffordlocksmiths.co.uk</t>
+          <t>keyrisestafford-locksmiths.co.uk</t>
         </is>
       </c>
     </row>
@@ -8017,7 +8017,7 @@
       <c r="L154" s="2" t="inlineStr"/>
       <c r="M154" s="2" t="inlineStr">
         <is>
-          <t>latchriselocksmithswalsall.co.uk</t>
+          <t>latchriselocksmiths-walsall.co.uk</t>
         </is>
       </c>
     </row>
@@ -8068,7 +8068,7 @@
       <c r="L155" s="2" t="inlineStr"/>
       <c r="M155" s="2" t="inlineStr">
         <is>
-          <t>locksprintwarwicklocksmith.co.uk</t>
+          <t>locksprint-warwicklocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -8119,7 +8119,7 @@
       <c r="L156" s="2" t="inlineStr"/>
       <c r="M156" s="2" t="inlineStr">
         <is>
-          <t>lockzonewolverhamptonlocksmith.co.uk</t>
+          <t>lockzone-wolverhampton-locksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -8170,7 +8170,7 @@
       <c r="L157" s="2" t="inlineStr"/>
       <c r="M157" s="2" t="inlineStr">
         <is>
-          <t>boltdashlocksmithworcester.co.uk</t>
+          <t>boltdashlocksmith-worcester.co.uk</t>
         </is>
       </c>
     </row>
@@ -8221,7 +8221,7 @@
       <c r="L158" s="2" t="inlineStr"/>
       <c r="M158" s="2" t="inlineStr">
         <is>
-          <t>boltriselocksmithbarnsley.co.uk</t>
+          <t>boltriselocksmith-barnsley.co.uk</t>
         </is>
       </c>
     </row>
@@ -8272,7 +8272,7 @@
       <c r="L159" s="2" t="inlineStr"/>
       <c r="M159" s="2" t="inlineStr">
         <is>
-          <t>lockquestharrogatelocksmith.co.uk</t>
+          <t>lockquest-harrogatelocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -8374,7 +8374,7 @@
       <c r="L161" s="2" t="inlineStr"/>
       <c r="M161" s="2" t="inlineStr">
         <is>
-          <t>keysquadmorleylocksmiths.co.uk</t>
+          <t>keysquadmorley-locksmiths.co.uk</t>
         </is>
       </c>
     </row>
@@ -8425,7 +8425,7 @@
       <c r="L162" s="2" t="inlineStr"/>
       <c r="M162" s="2" t="inlineStr">
         <is>
-          <t>lockriserotherhamlocksmith.co.uk</t>
+          <t>lockriserotherham-locksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -8527,7 +8527,7 @@
       <c r="L164" s="2" t="inlineStr"/>
       <c r="M164" s="2" t="inlineStr">
         <is>
-          <t>latchlinelocksmithsyork.co.uk</t>
+          <t>latchline-locksmiths-york.co.uk</t>
         </is>
       </c>
     </row>
@@ -8884,7 +8884,7 @@
       <c r="L171" s="2" t="inlineStr"/>
       <c r="M171" s="2" t="inlineStr">
         <is>
-          <t>latchquestlocksmithssouthshields.co.uk</t>
+          <t>latchquest-locksmithssouthshields.co.uk</t>
         </is>
       </c>
     </row>
@@ -9496,7 +9496,7 @@
       <c r="L183" s="2" t="inlineStr"/>
       <c r="M183" s="2" t="inlineStr">
         <is>
-          <t>keyservedewsburylocksmiths.co.uk</t>
+          <t>keyserve-dewsburylocksmiths.co.uk</t>
         </is>
       </c>
     </row>
@@ -9649,7 +9649,7 @@
       <c r="L186" s="2" t="inlineStr"/>
       <c r="M186" s="2" t="inlineStr">
         <is>
-          <t>keymateblackburnlocksmiths.co.uk</t>
+          <t>keymateblackburn-locksmiths.co.uk</t>
         </is>
       </c>
     </row>
@@ -9700,7 +9700,7 @@
       <c r="L187" s="2" t="inlineStr"/>
       <c r="M187" s="2" t="inlineStr">
         <is>
-          <t>latchnodelocksmithsburnley.co.uk</t>
+          <t>latchnodelocksmiths-burnley.co.uk</t>
         </is>
       </c>
     </row>
@@ -9751,7 +9751,7 @@
       <c r="L188" s="2" t="inlineStr"/>
       <c r="M188" s="2" t="inlineStr">
         <is>
-          <t>locknodeburylocksmith.co.uk</t>
+          <t>locknodebury-locksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -10567,7 +10567,7 @@
       <c r="L204" s="2" t="inlineStr"/>
       <c r="M204" s="2" t="inlineStr">
         <is>
-          <t>latchcorelocksmithssouthport.co.uk</t>
+          <t>latchcore-locksmiths-southport.co.uk</t>
         </is>
       </c>
     </row>
@@ -11026,7 +11026,7 @@
       <c r="L213" s="2" t="inlineStr"/>
       <c r="M213" s="2" t="inlineStr">
         <is>
-          <t>keynodescunthorpelocksmiths.co.uk</t>
+          <t>keynodescunthorpe-locksmiths.co.uk</t>
         </is>
       </c>
     </row>
@@ -11587,7 +11587,7 @@
       <c r="L224" s="2" t="inlineStr"/>
       <c r="M224" s="2" t="inlineStr">
         <is>
-          <t>keylinkhuddersfieldlocksmiths.co.uk</t>
+          <t>keylink-huddersfieldlocksmiths.co.uk</t>
         </is>
       </c>
     </row>
@@ -12148,7 +12148,7 @@
       <c r="L235" s="2" t="inlineStr"/>
       <c r="M235" s="2" t="inlineStr">
         <is>
-          <t>keycraftbirkenheadlocksmiths.co.uk</t>
+          <t>keycraft-birkenheadlocksmiths.co.uk</t>
         </is>
       </c>
     </row>
@@ -12301,7 +12301,7 @@
       <c r="L238" s="2" t="inlineStr"/>
       <c r="M238" s="2" t="inlineStr">
         <is>
-          <t>lockrouteellesmereportlocksmith.co.uk</t>
+          <t>lockroute-ellesmereport-locksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -12556,7 +12556,7 @@
       <c r="L243" s="2" t="inlineStr"/>
       <c r="M243" s="2" t="inlineStr">
         <is>
-          <t>lockdashsthelenslocksmith.co.uk</t>
+          <t>lockdashsthelens-locksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -12862,7 +12862,7 @@
       <c r="L249" s="2" t="inlineStr"/>
       <c r="M249" s="2" t="inlineStr">
         <is>
-          <t>boltquestlocksmithcrewe.co.uk</t>
+          <t>boltquest-locksmithcrewe.co.uk</t>
         </is>
       </c>
     </row>
@@ -13015,7 +13015,7 @@
       <c r="L252" s="2" t="inlineStr"/>
       <c r="M252" s="2" t="inlineStr">
         <is>
-          <t>locksmartsalelocksmith.co.uk</t>
+          <t>locksmartsale-locksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -13525,7 +13525,7 @@
       <c r="L262" s="2" t="inlineStr"/>
       <c r="M262" s="2" t="inlineStr">
         <is>
-          <t>lockservemansfieldlocksmith.co.uk</t>
+          <t>lockserve-mansfieldlocksmith.co.uk</t>
         </is>
       </c>
     </row>
@@ -14392,7 +14392,7 @@
       <c r="L279" s="2" t="inlineStr"/>
       <c r="M279" s="2" t="inlineStr">
         <is>
-          <t>keysmartcannocklocksmiths.co.uk</t>
+          <t>keysmartcannock-locksmiths.co.uk</t>
         </is>
       </c>
     </row>
@@ -14443,7 +14443,7 @@
       <c r="L280" s="2" t="inlineStr"/>
       <c r="M280" s="2" t="inlineStr">
         <is>
-          <t>latchgridlocksmithsnuneaton.co.uk</t>
+          <t>latchgridlocksmiths-nuneaton.co.uk</t>
         </is>
       </c>
     </row>
@@ -14647,7 +14647,7 @@
       <c r="L284" s="2" t="inlineStr"/>
       <c r="M284" s="2" t="inlineStr">
         <is>
-          <t>latchdashlocksmithswestbromwich.co.uk</t>
+          <t>latchdashlocksmiths-westbromwich.co.uk</t>
         </is>
       </c>
     </row>
@@ -15208,7 +15208,7 @@
       <c r="L295" s="2" t="inlineStr"/>
       <c r="M295" s="2" t="inlineStr">
         <is>
-          <t>latchservelocksmithskettering.co.uk</t>
+          <t>latchserve-locksmithskettering.co.uk</t>
         </is>
       </c>
     </row>
@@ -16585,7 +16585,7 @@
       <c r="L322" s="2" t="inlineStr"/>
       <c r="M322" s="2" t="inlineStr">
         <is>
-          <t>boltlinklocksmithwatford.co.uk</t>
+          <t>boltlink-locksmithwatford.co.uk</t>
         </is>
       </c>
     </row>
@@ -17605,7 +17605,7 @@
       <c r="L342" s="2" t="inlineStr"/>
       <c r="M342" s="2" t="inlineStr">
         <is>
-          <t>boltservelocksmithmargate.co.uk</t>
+          <t>boltserve-locksmithmargate.co.uk</t>
         </is>
       </c>
     </row>
@@ -17911,7 +17911,7 @@
       <c r="L348" s="2" t="inlineStr"/>
       <c r="M348" s="2" t="inlineStr">
         <is>
-          <t>keykinghighwycombelocksmiths.co.uk</t>
+          <t>keyking-highwycombelocksmiths.co.uk</t>
         </is>
       </c>
     </row>
@@ -18166,7 +18166,7 @@
       <c r="L353" s="2" t="inlineStr"/>
       <c r="M353" s="2" t="inlineStr">
         <is>
-          <t>keypeakswindonlocksmiths.co.uk</t>
+          <t>keypeakswindon-locksmiths.co.uk</t>
         </is>
       </c>
     </row>
@@ -18574,7 +18574,7 @@
       <c r="L361" s="2" t="inlineStr"/>
       <c r="M361" s="2" t="inlineStr">
         <is>
-          <t>keyrouterochesterlocksmiths.co.uk</t>
+          <t>keyroute-rochester-locksmiths.co.uk</t>
         </is>
       </c>
     </row>
@@ -18778,7 +18778,7 @@
       <c r="L365" s="2" t="inlineStr"/>
       <c r="M365" s="2" t="inlineStr">
         <is>
-          <t>boltnodelocksmithbracknell.co.uk</t>
+          <t>boltnodelocksmith-bracknell.co.uk</t>
         </is>
       </c>
     </row>
@@ -20818,7 +20818,7 @@
       <c r="L405" s="2" t="inlineStr"/>
       <c r="M405" s="2" t="inlineStr">
         <is>
-          <t>lockgridhovelocksmith.co.uk</t>
+          <t>lockgridhove-locksmith.co.uk</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Drop the brandlocksmith(s)-city domain shape
Reassigns the 14 domains using that pattern to the other hyphenation
styles; all replacements DNS-checked as available.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018qYwdxW5238hQ6ii9dUE6c
</commit_message>
<xml_diff>
--- a/data/locksmith-fleet/coverage-plan-final.xlsx
+++ b/data/locksmith-fleet/coverage-plan-final.xlsx
@@ -2471,7 +2471,7 @@
       </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>boltsmartlocksmith-runcorn.co.uk</t>
+          <t>boltsmartlocksmithruncorn.co.uk</t>
         </is>
       </c>
     </row>
@@ -2589,7 +2589,7 @@
       </c>
       <c r="M44" s="2" t="inlineStr">
         <is>
-          <t>boltpeaklocksmith-warrington.co.uk</t>
+          <t>boltpeaklocksmithwarrington.co.uk</t>
         </is>
       </c>
     </row>
@@ -3103,7 +3103,7 @@
       </c>
       <c r="M55" s="2" t="inlineStr">
         <is>
-          <t>latchsmartlocksmiths-farnborough.co.uk</t>
+          <t>latchsmart-locksmiths-farnborough.co.uk</t>
         </is>
       </c>
     </row>
@@ -3250,7 +3250,7 @@
       </c>
       <c r="M58" s="2" t="inlineStr">
         <is>
-          <t>boltgridlocksmith-hastings.co.uk</t>
+          <t>boltgridlocksmithhastings.co.uk</t>
         </is>
       </c>
     </row>
@@ -3485,7 +3485,7 @@
       </c>
       <c r="M63" s="2" t="inlineStr">
         <is>
-          <t>latchpeaklocksmiths-oxford.co.uk</t>
+          <t>latchpeak-locksmiths-oxford.co.uk</t>
         </is>
       </c>
     </row>
@@ -6538,7 +6538,7 @@
       <c r="L125" s="2" t="inlineStr"/>
       <c r="M125" s="2" t="inlineStr">
         <is>
-          <t>latchmatelocksmiths-stockport.co.uk</t>
+          <t>latchmatelocksmithsstockport.co.uk</t>
         </is>
       </c>
     </row>
@@ -7405,7 +7405,7 @@
       <c r="L142" s="2" t="inlineStr"/>
       <c r="M142" s="2" t="inlineStr">
         <is>
-          <t>boltmatelocksmith-gloucester.co.uk</t>
+          <t>boltmate-locksmithgloucester.co.uk</t>
         </is>
       </c>
     </row>
@@ -8017,7 +8017,7 @@
       <c r="L154" s="2" t="inlineStr"/>
       <c r="M154" s="2" t="inlineStr">
         <is>
-          <t>latchriselocksmiths-walsall.co.uk</t>
+          <t>latchrise-locksmithswalsall.co.uk</t>
         </is>
       </c>
     </row>
@@ -8170,7 +8170,7 @@
       <c r="L157" s="2" t="inlineStr"/>
       <c r="M157" s="2" t="inlineStr">
         <is>
-          <t>boltdashlocksmith-worcester.co.uk</t>
+          <t>boltdash-locksmith-worcester.co.uk</t>
         </is>
       </c>
     </row>
@@ -8221,7 +8221,7 @@
       <c r="L158" s="2" t="inlineStr"/>
       <c r="M158" s="2" t="inlineStr">
         <is>
-          <t>boltriselocksmith-barnsley.co.uk</t>
+          <t>boltrise-locksmith-barnsley.co.uk</t>
         </is>
       </c>
     </row>
@@ -9700,7 +9700,7 @@
       <c r="L187" s="2" t="inlineStr"/>
       <c r="M187" s="2" t="inlineStr">
         <is>
-          <t>latchnodelocksmiths-burnley.co.uk</t>
+          <t>latchnodelocksmithsburnley.co.uk</t>
         </is>
       </c>
     </row>
@@ -14443,7 +14443,7 @@
       <c r="L280" s="2" t="inlineStr"/>
       <c r="M280" s="2" t="inlineStr">
         <is>
-          <t>latchgridlocksmiths-nuneaton.co.uk</t>
+          <t>latchgrid-locksmiths-nuneaton.co.uk</t>
         </is>
       </c>
     </row>
@@ -14647,7 +14647,7 @@
       <c r="L284" s="2" t="inlineStr"/>
       <c r="M284" s="2" t="inlineStr">
         <is>
-          <t>latchdashlocksmiths-westbromwich.co.uk</t>
+          <t>latchdash-locksmithswestbromwich.co.uk</t>
         </is>
       </c>
     </row>
@@ -18778,7 +18778,7 @@
       <c r="L365" s="2" t="inlineStr"/>
       <c r="M365" s="2" t="inlineStr">
         <is>
-          <t>boltnodelocksmith-bracknell.co.uk</t>
+          <t>boltnode-locksmithbracknell.co.uk</t>
         </is>
       </c>
     </row>

</xml_diff>